<commit_message>
Actualización de datos y diccionario de sinergias - Abril 2026
</commit_message>
<xml_diff>
--- a/public/data/diccionario_sinergias_final.xlsx
+++ b/public/data/diccionario_sinergias_final.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C282"/>
+  <dimension ref="A1:C277"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -560,21 +560,21 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
+        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
       </c>
       <c r="B14" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>PREVENCIÓN Y EXTINCIÓN DE INCENDIOS PARA EQUIPOS DE PRIMERA INTERVENCIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C14" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Extinción Incendios, Incendios</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
+        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
       </c>
       <c r="B15" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="C15" t="str">
         <v>Puente Grúa, Grúa</v>
@@ -582,43 +582,43 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
       </c>
       <c r="B16" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="C16" t="str">
-        <v>Carretillas, PRL</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios de máquinas de mecanizado por arranque de viruta o por abrasión</v>
       </c>
       <c r="B17" t="str">
-        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>NIVEL BÁSICO PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA</v>
       </c>
       <c r="C17" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Metal, PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
+        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B18" t="str">
-        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C18" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Carretillas, PRL</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B19" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C19" t="str">
         <v>Carretillas, Seguridad</v>
@@ -626,43 +626,43 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
       </c>
       <c r="B20" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C20" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B21" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C21" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B22" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C22" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B23" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C23" t="str">
         <v>Espacios Confinados, Seguridad</v>
@@ -670,164 +670,164 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ALTURAS TELCO I</v>
+        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
       </c>
       <c r="B24" t="str">
-        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C24" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B25" t="str">
-        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN TRABAJOS EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C25" t="str">
-        <v>Carretillas</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
+        <v>ALTURAS TELCO I</v>
       </c>
       <c r="B26" t="str">
-        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
+        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C26" t="str">
-        <v>Carretillas</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B27" t="str">
-        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C27" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ESPACIOS CONFINADOS TELCO</v>
+        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
       </c>
       <c r="B28" t="str">
-        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
       </c>
       <c r="C28" t="str">
-        <v>Espacios Confinados</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="B29" t="str">
-        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
+        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="C29" t="str">
-        <v>Construcción, Nivel Básico</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios de máquinas de mecanizado por arranque de viruta o por abrasión</v>
+        <v>ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B30" t="str">
-        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
+        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C30" t="str">
-        <v>Metal, Nivel Básico</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
+        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
       </c>
       <c r="B31" t="str">
-        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
+        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C31" t="str">
-        <v>Carretillas</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PRIMEROS AUXILIOS</v>
+        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
       </c>
       <c r="B32" t="str">
-        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
+        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
       </c>
       <c r="C32" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
       </c>
       <c r="B33" t="str">
-        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
       </c>
       <c r="C33" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Metal, Nivel Básico</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
+        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B34" t="str">
-        <v>PRL EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C34" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
+        <v>PRIMEROS AUXILIOS</v>
       </c>
       <c r="B35" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C35" t="str">
-        <v>Metal, PRL</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
+        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
       </c>
       <c r="B36" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C36" t="str">
-        <v>Metal, PRL</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
       </c>
       <c r="B37" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C37" t="str">
-        <v>Metal, PRL</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
+        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
       </c>
       <c r="B38" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C38" t="str">
         <v>Metal, PRL</v>
@@ -835,10 +835,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
       </c>
       <c r="B39" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C39" t="str">
         <v>Metal, PRL</v>
@@ -846,87 +846,87 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
       </c>
       <c r="B40" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C40" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
       </c>
       <c r="B41" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C41" t="str">
-        <v>Carretillas</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
       </c>
       <c r="B42" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C42" t="str">
-        <v>Soldadura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>RECICLAJE  ALTURAS TELCO I</v>
+        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
       </c>
       <c r="B43" t="str">
-        <v>RECICLAJE ALTURAS TELCO II. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C43" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B44" t="str">
-        <v>RECICLAJE DE CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C44" t="str">
-        <v>Carretillas</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
+        <v>RECICLAJE  ALTURAS TELCO I</v>
       </c>
       <c r="B45" t="str">
-        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
+        <v>RECICLAJE ALTURAS TELCO II. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C45" t="str">
-        <v>Amianto</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
       </c>
       <c r="B46" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
       </c>
       <c r="C46" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
+        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B47" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C15- INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C47" t="str">
         <v>Riesgo Eléctrico</v>
@@ -934,32 +934,32 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
       </c>
       <c r="B48" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C15- INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C48" t="str">
-        <v>Soldadura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B49" t="str">
-        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C49" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
       </c>
       <c r="B50" t="str">
-        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C50" t="str">
         <v>Riesgo Eléctrico</v>
@@ -967,10 +967,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
+        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B51" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C51" t="str">
         <v>Riesgo Eléctrico</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
+        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B52" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C52" t="str">
         <v>Riesgo Eléctrico</v>
@@ -989,10 +989,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>RIESGO ELÉCTRICO TELCO</v>
+        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
       </c>
       <c r="B53" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C53" t="str">
         <v>Riesgo Eléctrico</v>
@@ -1000,10 +1000,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
+        <v>RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B54" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C54" t="str">
         <v>Riesgo Eléctrico</v>
@@ -1011,54 +1011,54 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>FORMACIÓN PREVENTIVA DE RECICLAJE PARA OPERARIOS EN TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR SEGÚN UNE 171370-1</v>
+        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
       </c>
       <c r="B55" t="str">
-        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C55" t="str">
-        <v>Amianto</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
+        <v>FORMACIÓN PREVENTIVA DE RECICLAJE PARA OPERARIOS EN TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR SEGÚN UNE 171370-1</v>
       </c>
       <c r="B56" t="str">
-        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C56" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
       </c>
       <c r="B57" t="str">
-        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
+        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C57" t="str">
-        <v>Construcción</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="B58" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
       </c>
       <c r="C58" t="str">
-        <v>Metal</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
+        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B59" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C59" t="str">
         <v>Metal</v>
@@ -1066,10 +1066,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B60" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C60" t="str">
         <v>Metal</v>
@@ -1077,13 +1077,13 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Mantenimiento de maquinaria y vehículos  en obras de construcción</v>
+        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="B61" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C61" t="str">
-        <v>Construcción</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="62">
@@ -1091,7 +1091,7 @@
         <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B62" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C62" t="str">
         <v>Metal</v>
@@ -1099,18 +1099,18 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>Mantenimiento de maquinaria y vehículos  en obras de construcción</v>
       </c>
       <c r="B63" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="C63" t="str">
-        <v>Metal</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>OTROS OFICIOS DEL METAL</v>
+        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B64" t="str">
         <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
@@ -1121,7 +1121,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B65" t="str">
         <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
@@ -1132,7 +1132,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B66" t="str">
         <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
@@ -1143,7 +1143,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B67" t="str">
         <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
@@ -1154,32 +1154,32 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Mantenimiento de maquinaria y vehículos en obras de construcción</v>
+        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B68" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C68" t="str">
-        <v>Construcción</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
+        <v>Mantenimiento de maquinaria y vehículos en obras de construcción</v>
       </c>
       <c r="B69" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="C69" t="str">
-        <v>Incendios</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
+        <v>OPERARIOS DE INSTALACIÓN Y MANTENIMIENTO DE EQUIPOS CONTRA INCENDIOS</v>
       </c>
       <c r="B70" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
       </c>
       <c r="C70" t="str">
         <v>Incendios</v>
@@ -1187,18 +1187,18 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>ACOSO LABORAL Y SEXUAL</v>
+        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B71" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
       </c>
       <c r="C71" t="str">
-        <v>—</v>
+        <v>Incendios</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>ADMINISTRATIVOS</v>
+        <v>ACOSO LABORAL Y SEXUAL</v>
       </c>
       <c r="B72" t="str">
         <v/>
@@ -1209,7 +1209,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>ALBAÑILERÍA</v>
+        <v>ADMINISTRATIVOS</v>
       </c>
       <c r="B73" t="str">
         <v/>
@@ -1220,7 +1220,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Campaña Allive 80.0 Fase II-Técnico de Prevención por un día-EL ALTO</v>
+        <v>ALBAÑILERÍA</v>
       </c>
       <c r="B74" t="str">
         <v/>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CARPINTERÍA METÁLICA</v>
+        <v>Campaña Allive 80.0 Fase II-Técnico de Prevención por un día-EL ALTO</v>
       </c>
       <c r="B75" t="str">
         <v/>
@@ -1242,29 +1242,29 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CONDUCCIÓN SEGURA</v>
+        <v>CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B76" t="str">
         <v/>
       </c>
       <c r="C76" t="str">
-        <v>Conducción</v>
+        <v>—</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CONDUCTORES Y TRANSPORTISTAS</v>
+        <v>CONDUCCIÓN SEGURA</v>
       </c>
       <c r="B77" t="str">
         <v/>
       </c>
       <c r="C77" t="str">
-        <v>—</v>
+        <v>Conducción</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>CONDUCTORES Y TRANSPORTISTAS</v>
       </c>
       <c r="B78" t="str">
         <v/>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="B79" t="str">
         <v/>
@@ -1286,29 +1286,29 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
+        <v>CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="B80" t="str">
         <v/>
       </c>
       <c r="C80" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
       </c>
       <c r="B81" t="str">
         <v/>
       </c>
       <c r="C81" t="str">
-        <v>—</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>ENCOFRADOS</v>
+        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="B82" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
+        <v>ENCOFRADOS</v>
       </c>
       <c r="B83" t="str">
         <v/>
@@ -1330,7 +1330,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>ESTABILIZACIÓN DE EXPLANADAS Y EXTENDIDO DE FIRMES</v>
+        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
       </c>
       <c r="B84" t="str">
         <v/>
@@ -1341,10 +1341,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v/>
+        <v>ESTABILIZACIÓN DE EXPLANADAS Y EXTENDIDO DE FIRMES</v>
       </c>
       <c r="B85" t="str">
-        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
+        <v/>
       </c>
       <c r="C85" t="str">
         <v>—</v>
@@ -1352,10 +1352,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>FERRALLADO</v>
+        <v/>
       </c>
       <c r="B86" t="str">
-        <v/>
+        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
       </c>
       <c r="C86" t="str">
         <v>—</v>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>FERRALLADO</v>
       </c>
       <c r="B87" t="str">
         <v/>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B88" t="str">
         <v/>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>FORMACIÓN DE INTERVENCIÓN EN EQUIPOS Y MÁQUINAS</v>
+        <v>FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="B89" t="str">
         <v/>
@@ -1396,7 +1396,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
+        <v>FORMACIÓN DE INTERVENCIÓN EN EQUIPOS Y MÁQUINAS</v>
       </c>
       <c r="B90" t="str">
         <v/>
@@ -1407,24 +1407,24 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
+        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
       </c>
       <c r="B91" t="str">
         <v/>
       </c>
       <c r="C91" t="str">
-        <v>Grúa, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>FORMACIÓN ESPECÍFICA OFICIOS GRUPO 3</v>
+        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
       </c>
       <c r="B92" t="str">
         <v/>
       </c>
       <c r="C92" t="str">
-        <v>—</v>
+        <v>Grúa, Seguridad</v>
       </c>
     </row>
     <row r="93">
@@ -1550,18 +1550,18 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
+        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
       </c>
       <c r="B104" t="str">
         <v/>
       </c>
       <c r="C104" t="str">
-        <v>Espacios Confinados</v>
+        <v>—</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
+        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B105" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
       </c>
       <c r="B106" t="str">
         <v/>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
+        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B107" t="str">
         <v/>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>MANIPULACION DE ALIMENTOS</v>
       </c>
       <c r="B108" t="str">
         <v/>
@@ -1605,10 +1605,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>MANIPULACION DE ALIMENTOS</v>
+        <v/>
       </c>
       <c r="B109" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS</v>
       </c>
       <c r="C109" t="str">
         <v>—</v>
@@ -1619,7 +1619,7 @@
         <v/>
       </c>
       <c r="B110" t="str">
-        <v>MANIPULADOR DE ALIMENTOS</v>
+        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
       </c>
       <c r="C110" t="str">
         <v>—</v>
@@ -1627,10 +1627,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v/>
+        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B111" t="str">
-        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
+        <v/>
       </c>
       <c r="C111" t="str">
         <v>—</v>
@@ -1638,7 +1638,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B112" t="str">
         <v/>
@@ -1649,7 +1649,7 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
+        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B113" t="str">
         <v/>
@@ -1660,29 +1660,29 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>MEDIDAS DE EMERGENCIA</v>
       </c>
       <c r="B114" t="str">
         <v/>
       </c>
       <c r="C114" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>MEDIDAS DE EMERGENCIA</v>
+        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="B115" t="str">
         <v/>
       </c>
       <c r="C115" t="str">
-        <v>Emergencias</v>
+        <v>—</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>MONTAJE ANDAMIOS APOYADOS</v>
       </c>
       <c r="B116" t="str">
         <v/>
@@ -1693,7 +1693,7 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>MONTAJE ANDAMIOS APOYADOS</v>
+        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
       </c>
       <c r="B117" t="str">
         <v/>
@@ -1704,10 +1704,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
+        <v/>
       </c>
       <c r="B118" t="str">
-        <v/>
+        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C118" t="str">
         <v>—</v>
@@ -1715,51 +1715,51 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v/>
+        <v>NIVEL BÁSICO EN PREVENCIÓN DE RIESGOS LABORALES 50 H</v>
       </c>
       <c r="B119" t="str">
-        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C119" t="str">
-        <v>—</v>
+        <v>PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>NIVEL BÁSICO EN PREVENCIÓN DE RIESGOS LABORALES 50 H</v>
+        <v>OPERACIONES TELCO</v>
       </c>
       <c r="B120" t="str">
         <v/>
       </c>
       <c r="C120" t="str">
-        <v>PRL, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>OPERACIONES TELCO</v>
+        <v>OPERADOR DE CAMIÓN GRÚA</v>
       </c>
       <c r="B121" t="str">
         <v/>
       </c>
       <c r="C121" t="str">
-        <v>—</v>
+        <v>Grúa</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>OPERADOR DE CAMIÓN GRÚA</v>
+        <v>OPERADOR DE PALA CARGADORA</v>
       </c>
       <c r="B122" t="str">
         <v/>
       </c>
       <c r="C122" t="str">
-        <v>Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>OPERADOR DE PALA CARGADORA</v>
+        <v>OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B123" t="str">
         <v/>
@@ -1770,29 +1770,29 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>OPERADORES DE APARATOS ELEVADORES</v>
+        <v>OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="B124" t="str">
         <v/>
       </c>
       <c r="C124" t="str">
-        <v>—</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>OPERADORES DE PUENTE-GRÚA</v>
+        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B125" t="str">
         <v/>
       </c>
       <c r="C125" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B126" t="str">
         <v/>
@@ -1803,7 +1803,7 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
       </c>
       <c r="B127" t="str">
         <v/>
@@ -1814,7 +1814,7 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
+        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
       </c>
       <c r="B128" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B129" t="str">
         <v/>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B130" t="str">
         <v/>
@@ -1847,7 +1847,7 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B131" t="str">
         <v/>
@@ -1858,7 +1858,7 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
       </c>
       <c r="B132" t="str">
         <v/>
@@ -1869,7 +1869,7 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v>OTRO TIPO DE INSTALACIONES</v>
       </c>
       <c r="B133" t="str">
         <v/>
@@ -1880,7 +1880,7 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>OTRO TIPO DE INSTALACIONES</v>
+        <v>PINTURA</v>
       </c>
       <c r="B134" t="str">
         <v/>
@@ -1891,95 +1891,95 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>PINTURA</v>
+        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
       </c>
       <c r="B135" t="str">
         <v/>
       </c>
       <c r="C135" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
       </c>
       <c r="B136" t="str">
         <v/>
       </c>
       <c r="C136" t="str">
-        <v>Emergencias</v>
+        <v>PEMP, Seguridad</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
+        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
       </c>
       <c r="B137" t="str">
         <v/>
       </c>
       <c r="C137" t="str">
-        <v>PEMP, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
+        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
       </c>
       <c r="B138" t="str">
         <v/>
       </c>
       <c r="C138" t="str">
-        <v>—</v>
+        <v>Ergonomía, PRL</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
       </c>
       <c r="B139" t="str">
         <v/>
       </c>
       <c r="C139" t="str">
-        <v>Ergonomía, PRL</v>
+        <v>Grúa, PRL</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
+        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B140" t="str">
         <v/>
       </c>
       <c r="C140" t="str">
-        <v>Grúa, PRL</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
       </c>
       <c r="B141" t="str">
         <v/>
       </c>
       <c r="C141" t="str">
-        <v>ATEX, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES EN TRABAJOS CON RIESGO DE EXPOSICIÓN A AMIANTO</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
       </c>
       <c r="B142" t="str">
         <v/>
       </c>
       <c r="C142" t="str">
-        <v>Amianto, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
+        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
       </c>
       <c r="B143" t="str">
         <v/>
@@ -1990,90 +1990,90 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
+        <v/>
       </c>
       <c r="B144" t="str">
-        <v/>
+        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C144" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
+        <v>Primeros Auxilios en Equipos de Emergencia</v>
       </c>
       <c r="B145" t="str">
         <v/>
       </c>
       <c r="C145" t="str">
-        <v>PRL</v>
+        <v>Primeros Auxilios, Emergencias</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v/>
+        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
       </c>
       <c r="B146" t="str">
-        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C146" t="str">
-        <v>—</v>
+        <v>Primeros Auxilios, Emergencias</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Primeros Auxilios en Equipos de Emergencia</v>
+        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
       </c>
       <c r="B147" t="str">
         <v/>
       </c>
       <c r="C147" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>Manipulación Cargas, PRL</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
+        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B148" t="str">
         <v/>
       </c>
       <c r="C148" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
+        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B149" t="str">
         <v/>
       </c>
       <c r="C149" t="str">
-        <v>Manipulación Cargas, PRL</v>
+        <v>PEMP, Plataformas, PRL</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B150" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C150" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B151" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C151" t="str">
-        <v>PEMP, Plataformas, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="152">
@@ -2081,7 +2081,7 @@
         <v/>
       </c>
       <c r="B152" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C152" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="B153" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C153" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2103,7 +2103,7 @@
         <v/>
       </c>
       <c r="B154" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C154" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="B155" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C155" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2125,7 +2125,7 @@
         <v/>
       </c>
       <c r="B156" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C156" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2136,7 +2136,7 @@
         <v/>
       </c>
       <c r="B157" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C157" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2147,7 +2147,7 @@
         <v/>
       </c>
       <c r="B158" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C158" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2158,7 +2158,7 @@
         <v/>
       </c>
       <c r="B159" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C159" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2169,7 +2169,7 @@
         <v/>
       </c>
       <c r="B160" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C160" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2180,7 +2180,7 @@
         <v/>
       </c>
       <c r="B161" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C161" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2191,7 +2191,7 @@
         <v/>
       </c>
       <c r="B162" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C162" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2202,7 +2202,7 @@
         <v/>
       </c>
       <c r="B163" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C163" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2213,7 +2213,7 @@
         <v/>
       </c>
       <c r="B164" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C164" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2224,7 +2224,7 @@
         <v/>
       </c>
       <c r="B165" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C165" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2232,150 +2232,150 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v/>
+        <v>PRL SEGURIDAD VIAL</v>
       </c>
       <c r="B166" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C166" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL, Seguridad</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v/>
+        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
       </c>
       <c r="B167" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v/>
       </c>
       <c r="C167" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v/>
+        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
       </c>
       <c r="B168" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v/>
       </c>
       <c r="C168" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v/>
+        <v>PRODQUIM/000</v>
       </c>
       <c r="B169" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="C169" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>PRL SEGURIDAD VIAL</v>
+        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B170" t="str">
         <v/>
       </c>
       <c r="C170" t="str">
-        <v>PRL, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
+        <v/>
       </c>
       <c r="B171" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C171" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
+        <v/>
       </c>
       <c r="B172" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C172" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>PRODQUIM/000</v>
+        <v/>
       </c>
       <c r="B173" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C173" t="str">
-        <v>—</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B174" t="str">
         <v/>
       </c>
       <c r="C174" t="str">
-        <v>—</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v/>
+        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B175" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C175" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v/>
+        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B176" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C176" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B177" t="str">
         <v/>
       </c>
       <c r="C177" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
+        <v>RECICLAJE PARA FERRALLADO</v>
       </c>
       <c r="B178" t="str">
         <v/>
       </c>
       <c r="C178" t="str">
-        <v>Espacios Confinados</v>
+        <v>—</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B179" t="str">
         <v/>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>RECICLAJE PARA FERRALLADO</v>
+        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B180" t="str">
         <v/>
@@ -2397,7 +2397,7 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B181" t="str">
         <v/>
@@ -2408,7 +2408,7 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>RECICLAJE PARA INSTALACIÓN DE ASCENSORES</v>
+        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B182" t="str">
         <v/>
@@ -2419,7 +2419,7 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B183" t="str">
         <v/>
@@ -2430,7 +2430,7 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B184" t="str">
         <v/>
@@ -2441,29 +2441,29 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>RECICLAJE PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B185" t="str">
         <v/>
       </c>
       <c r="C185" t="str">
-        <v>—</v>
+        <v>PEMP, Plataformas</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>RECICLAJE PARA OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="B186" t="str">
         <v/>
       </c>
       <c r="C186" t="str">
-        <v>—</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B187" t="str">
         <v/>
@@ -2474,29 +2474,29 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>RECICLAJE PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B188" t="str">
         <v/>
       </c>
       <c r="C188" t="str">
-        <v>PEMP, Plataformas</v>
+        <v>—</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>RECICLAJE PARA OPERADORES DE PUENTE-GRÚA</v>
+        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B189" t="str">
         <v/>
       </c>
       <c r="C189" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
       </c>
       <c r="B190" t="str">
         <v/>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B191" t="str">
         <v/>
@@ -2518,35 +2518,35 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="B192" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C192" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v/>
       </c>
       <c r="B193" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C193" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="B194" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C194" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="195">
@@ -2554,7 +2554,7 @@
         <v/>
       </c>
       <c r="B195" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C195" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2565,7 +2565,7 @@
         <v/>
       </c>
       <c r="B196" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C196" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2576,7 +2576,7 @@
         <v/>
       </c>
       <c r="B197" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C197" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2584,40 +2584,40 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v/>
+        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
       </c>
       <c r="B198" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C198" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v/>
+        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B199" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v/>
       </c>
       <c r="C199" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v/>
+        <v>REVESTIMIENTO DE YESO</v>
       </c>
       <c r="B200" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="C200" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
+        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
       </c>
       <c r="B201" t="str">
         <v/>
@@ -2628,46 +2628,46 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
       </c>
       <c r="B202" t="str">
         <v/>
       </c>
       <c r="C202" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>REVESTIMIENTO DE YESO</v>
+        <v/>
       </c>
       <c r="B203" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20  HORAS): CIMENTACIONES ESPECIALES, SONDEOS Y PERFORACIONES</v>
       </c>
       <c r="C203" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
+        <v/>
       </c>
       <c r="B204" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C204" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
+        <v/>
       </c>
       <c r="B205" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C205" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="206">
@@ -2675,7 +2675,7 @@
         <v/>
       </c>
       <c r="B206" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C206" t="str">
         <v>Construcción, PRL</v>
@@ -2686,7 +2686,7 @@
         <v/>
       </c>
       <c r="B207" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C207" t="str">
         <v>Construcción, PRL</v>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="B208" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="C208" t="str">
         <v>Construcción, PRL</v>
@@ -2708,7 +2708,7 @@
         <v/>
       </c>
       <c r="B209" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C209" t="str">
         <v>Construcción, PRL</v>
@@ -2719,7 +2719,7 @@
         <v/>
       </c>
       <c r="B210" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C210" t="str">
         <v>Construcción, PRL</v>
@@ -2730,7 +2730,7 @@
         <v/>
       </c>
       <c r="B211" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
       </c>
       <c r="C211" t="str">
         <v>Construcción, PRL</v>
@@ -2741,7 +2741,7 @@
         <v/>
       </c>
       <c r="B212" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
       </c>
       <c r="C212" t="str">
         <v>Construcción, PRL</v>
@@ -2752,7 +2752,7 @@
         <v/>
       </c>
       <c r="B213" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C213" t="str">
         <v>Construcción, PRL</v>
@@ -2763,7 +2763,7 @@
         <v/>
       </c>
       <c r="B214" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C214" t="str">
         <v>Construcción, PRL</v>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="B215" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C215" t="str">
         <v>Construcción, PRL</v>
@@ -2785,7 +2785,7 @@
         <v/>
       </c>
       <c r="B216" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C216" t="str">
         <v>Construcción, PRL</v>
@@ -2796,7 +2796,7 @@
         <v/>
       </c>
       <c r="B217" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C217" t="str">
         <v>Construcción, PRL</v>
@@ -2807,7 +2807,7 @@
         <v/>
       </c>
       <c r="B218" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C218" t="str">
         <v>Construcción, PRL</v>
@@ -2818,7 +2818,7 @@
         <v/>
       </c>
       <c r="B219" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C219" t="str">
         <v>Construcción, PRL</v>
@@ -2829,7 +2829,7 @@
         <v/>
       </c>
       <c r="B220" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CIMENTACIONES ESPECIALES, SONDEOS Y PERFORACIONES</v>
       </c>
       <c r="C220" t="str">
         <v>Construcción, PRL</v>
@@ -2840,7 +2840,7 @@
         <v/>
       </c>
       <c r="B221" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C221" t="str">
         <v>Construcción, PRL</v>
@@ -2851,7 +2851,7 @@
         <v/>
       </c>
       <c r="B222" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C222" t="str">
         <v>Construcción, PRL</v>
@@ -2862,7 +2862,7 @@
         <v/>
       </c>
       <c r="B223" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="C223" t="str">
         <v>Construcción, PRL</v>
@@ -2873,7 +2873,7 @@
         <v/>
       </c>
       <c r="B224" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C224" t="str">
         <v>Construcción, PRL</v>
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="B225" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C225" t="str">
         <v>Construcción, PRL</v>
@@ -2895,7 +2895,7 @@
         <v/>
       </c>
       <c r="B226" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
       </c>
       <c r="C226" t="str">
         <v>Construcción, PRL</v>
@@ -2906,7 +2906,7 @@
         <v/>
       </c>
       <c r="B227" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
       </c>
       <c r="C227" t="str">
         <v>Construcción, PRL</v>
@@ -2917,7 +2917,7 @@
         <v/>
       </c>
       <c r="B228" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C228" t="str">
         <v>Construcción, PRL</v>
@@ -2928,7 +2928,7 @@
         <v/>
       </c>
       <c r="B229" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C229" t="str">
         <v>Construcción, PRL</v>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="B230" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C230" t="str">
         <v>Construcción, PRL</v>
@@ -2950,7 +2950,7 @@
         <v/>
       </c>
       <c r="B231" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C231" t="str">
         <v>Construcción, PRL</v>
@@ -2961,7 +2961,7 @@
         <v/>
       </c>
       <c r="B232" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C232" t="str">
         <v>Construcción, PRL</v>
@@ -2972,10 +2972,10 @@
         <v/>
       </c>
       <c r="B233" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C233" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="234">
@@ -2983,10 +2983,10 @@
         <v/>
       </c>
       <c r="B234" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): MANDOS INTERMEDIOS</v>
       </c>
       <c r="C234" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="235">
@@ -2994,10 +2994,10 @@
         <v/>
       </c>
       <c r="B235" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C235" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="236">
@@ -3005,7 +3005,7 @@
         <v/>
       </c>
       <c r="B236" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C236" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3016,7 +3016,7 @@
         <v/>
       </c>
       <c r="B237" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): MANDOS INTERMEDIOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C237" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3027,7 +3027,7 @@
         <v/>
       </c>
       <c r="B238" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C238" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3038,7 +3038,7 @@
         <v/>
       </c>
       <c r="B239" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCIÓN Y MANTENIMIENTO DE VÍAS FÉRREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C239" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3049,7 +3049,7 @@
         <v/>
       </c>
       <c r="B240" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C240" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3060,7 +3060,7 @@
         <v/>
       </c>
       <c r="B241" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C241" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3071,7 +3071,7 @@
         <v/>
       </c>
       <c r="B242" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C242" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="B243" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C243" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3093,7 +3093,7 @@
         <v/>
       </c>
       <c r="B244" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C244" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3104,7 +3104,7 @@
         <v/>
       </c>
       <c r="B245" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C245" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3112,95 +3112,95 @@
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v/>
+        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
       </c>
       <c r="B246" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCIÓN Y MANTENIMIENTO DE VÍAS FÉRREAS</v>
+        <v/>
       </c>
       <c r="C246" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
       </c>
       <c r="B247" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v/>
       </c>
       <c r="C247" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
       </c>
       <c r="B248" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C248" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
       </c>
       <c r="B249" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C249" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
       </c>
       <c r="B250" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C250" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
+        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA. RECICLAJE</v>
       </c>
       <c r="B251" t="str">
         <v/>
       </c>
       <c r="C251" t="str">
-        <v>Seguridad</v>
+        <v>Puente Grúa, Grúa, Seguridad</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
+        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B252" t="str">
         <v/>
       </c>
       <c r="C252" t="str">
-        <v>Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
+        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
       </c>
       <c r="B253" t="str">
         <v/>
       </c>
       <c r="C253" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
+        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B254" t="str">
         <v/>
@@ -3211,161 +3211,161 @@
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
       </c>
       <c r="B255" t="str">
         <v/>
       </c>
       <c r="C255" t="str">
-        <v>Seguridad</v>
+        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA. RECICLAJE</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
       </c>
       <c r="B256" t="str">
         <v/>
       </c>
       <c r="C256" t="str">
-        <v>Puente Grúa, Grúa, Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
       </c>
       <c r="B257" t="str">
         <v/>
       </c>
       <c r="C257" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
       </c>
       <c r="B258" t="str">
         <v/>
       </c>
       <c r="C258" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
       </c>
       <c r="B259" t="str">
         <v/>
       </c>
       <c r="C259" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
+        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
       </c>
       <c r="B260" t="str">
         <v/>
       </c>
       <c r="C260" t="str">
-        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
+        <v>Riesgo Químico, Seguridad</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
+        <v>SEGURIDAD Y SALUD EN EL MANEJO DE TRANSPALETAS ELÉCTRICAS Y TRANSPALETAS MANUALES</v>
       </c>
       <c r="B261" t="str">
         <v/>
       </c>
       <c r="C261" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
+        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
       </c>
       <c r="B262" t="str">
         <v/>
       </c>
       <c r="C262" t="str">
-        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
+        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
       </c>
       <c r="B263" t="str">
         <v/>
       </c>
       <c r="C263" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Grúa, Conducción Vehículos</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
+        <v>SOLADOS Y ALICATADOS</v>
       </c>
       <c r="B264" t="str">
         <v/>
       </c>
       <c r="C264" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B265" t="str">
         <v/>
       </c>
       <c r="C265" t="str">
-        <v>Riesgo Químico, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE TRANSPALETAS ELÉCTRICAS Y TRANSPALETAS MANUALES</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B266" t="str">
         <v/>
       </c>
       <c r="C266" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
+        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B267" t="str">
         <v/>
       </c>
       <c r="C267" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
+        <v>TEÓRICO-PRÁCTICO DE MONTAJE DE PUNTOS DE ANCLAJE Y LÍNEAS DE VIDA PROVISIONALES</v>
       </c>
       <c r="B268" t="str">
         <v/>
       </c>
       <c r="C268" t="str">
-        <v>Grúa, Conducción Vehículos</v>
+        <v>—</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>SOLADOS Y ALICATADOS</v>
+        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
       </c>
       <c r="B269" t="str">
         <v/>
@@ -3376,29 +3376,29 @@
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v>TRABAJOS DE ARQUEOLOGÍA</v>
       </c>
       <c r="B270" t="str">
         <v/>
       </c>
       <c r="C270" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B271" t="str">
         <v/>
       </c>
       <c r="C271" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
       </c>
       <c r="B272" t="str">
         <v/>
@@ -3409,7 +3409,7 @@
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>TEÓRICO-PRÁCTICO DE MONTAJE DE PUNTOS DE ANCLAJE Y LÍNEAS DE VIDA PROVISIONALES</v>
+        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
       </c>
       <c r="B273" t="str">
         <v/>
@@ -3420,29 +3420,29 @@
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
+        <v>TRABAJOS DE SOLDADURA</v>
       </c>
       <c r="B274" t="str">
         <v/>
       </c>
       <c r="C274" t="str">
-        <v>—</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>TRABAJOS DE ARQUEOLOGÍA</v>
+        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
       </c>
       <c r="B275" t="str">
         <v/>
       </c>
       <c r="C275" t="str">
-        <v>—</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
       </c>
       <c r="B276" t="str">
         <v/>
@@ -3453,73 +3453,18 @@
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
       </c>
       <c r="B277" t="str">
         <v/>
       </c>
       <c r="C277" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="str">
-        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
-      </c>
-      <c r="B278" t="str">
-        <v/>
-      </c>
-      <c r="C278" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="str">
-        <v>TRABAJOS DE SOLDADURA</v>
-      </c>
-      <c r="B279" t="str">
-        <v/>
-      </c>
-      <c r="C279" t="str">
-        <v>Soldadura</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="str">
-        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
-      </c>
-      <c r="B280" t="str">
-        <v/>
-      </c>
-      <c r="C280" t="str">
-        <v>Trabajos en Altura</v>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
-      </c>
-      <c r="B281" t="str">
-        <v/>
-      </c>
-      <c r="C281" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
-      </c>
-      <c r="B282" t="str">
-        <v/>
-      </c>
-      <c r="C282" t="str">
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C282"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C277"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización de datos y diccionario de sinergias - 20 Abril 2026
</commit_message>
<xml_diff>
--- a/public/data/diccionario_sinergias_final.xlsx
+++ b/public/data/diccionario_sinergias_final.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C277"/>
+  <dimension ref="A1:C269"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -560,21 +560,21 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
+        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
       </c>
       <c r="B14" t="str">
-        <v>PREVENCIÓN Y EXTINCIÓN DE INCENDIOS PARA EQUIPOS DE PRIMERA INTERVENCIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="C14" t="str">
-        <v>Extinción Incendios, Incendios</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
+        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
       </c>
       <c r="B15" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="C15" t="str">
         <v>Puente Grúa, Grúa</v>
@@ -582,65 +582,65 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
       </c>
       <c r="B16" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>NIVEL BÁSICO PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA</v>
       </c>
       <c r="C16" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Metal, PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios de máquinas de mecanizado por arranque de viruta o por abrasión</v>
+        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B17" t="str">
-        <v>NIVEL BÁSICO PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C17" t="str">
-        <v>Metal, PRL, Nivel Básico</v>
+        <v>Carretillas, PRL</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B18" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C18" t="str">
-        <v>Carretillas, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
       </c>
       <c r="B19" t="str">
-        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C19" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B20" t="str">
-        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C20" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B21" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C21" t="str">
         <v>Carretillas, Seguridad</v>
@@ -648,230 +648,230 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B22" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C22" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
       </c>
       <c r="B23" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C23" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
+        <v>ALTURAS TELCO I</v>
       </c>
       <c r="B24" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C24" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B25" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C25" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ALTURAS TELCO I</v>
+        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
       </c>
       <c r="B26" t="str">
-        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
+        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
       </c>
       <c r="C26" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="B27" t="str">
-        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
+        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="C27" t="str">
-        <v>Carretillas</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
+        <v>ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B28" t="str">
-        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
+        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C28" t="str">
-        <v>Carretillas</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
       </c>
       <c r="B29" t="str">
-        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
       </c>
       <c r="C29" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ESPACIOS CONFINADOS TELCO</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
       </c>
       <c r="B30" t="str">
-        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
+        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
       </c>
       <c r="C30" t="str">
-        <v>Espacios Confinados</v>
+        <v>Metal, Nivel Básico</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
+        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B31" t="str">
-        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C31" t="str">
-        <v>Espacios Confinados</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
+        <v>PRIMEROS AUXILIOS</v>
       </c>
       <c r="B32" t="str">
-        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
+        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C32" t="str">
-        <v>Construcción, Nivel Básico</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
+        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
       </c>
       <c r="B33" t="str">
-        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
+        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C33" t="str">
-        <v>Metal, Nivel Básico</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
+        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
       </c>
       <c r="B34" t="str">
-        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C34" t="str">
-        <v>Carretillas</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PRIMEROS AUXILIOS</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
       </c>
       <c r="B35" t="str">
-        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C35" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
       </c>
       <c r="B36" t="str">
-        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C36" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
+        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
       </c>
       <c r="B37" t="str">
-        <v>PRL EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C37" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
+        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
       </c>
       <c r="B38" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C38" t="str">
-        <v>Metal, PRL</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
+        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B39" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C39" t="str">
-        <v>Metal, PRL</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
       </c>
       <c r="B40" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C40" t="str">
-        <v>Metal, PRL</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
+        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
       </c>
       <c r="B41" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
       </c>
       <c r="C41" t="str">
-        <v>Metal, PRL</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
+        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B42" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C42" t="str">
         <v>Riesgo Eléctrico</v>
@@ -879,21 +879,21 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
+        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
       </c>
       <c r="B43" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C15- INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C43" t="str">
-        <v>Carretillas</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B44" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C44" t="str">
         <v>Soldadura</v>
@@ -901,32 +901,32 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>RECICLAJE  ALTURAS TELCO I</v>
+        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
       </c>
       <c r="B45" t="str">
-        <v>RECICLAJE ALTURAS TELCO II. TEÓRICO-PRÁCTICO</v>
+        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C45" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
+        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B46" t="str">
-        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
+        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C46" t="str">
-        <v>Amianto</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B47" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C47" t="str">
         <v>Riesgo Eléctrico</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
+        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
       </c>
       <c r="B48" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C15- INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C48" t="str">
         <v>Riesgo Eléctrico</v>
@@ -945,21 +945,21 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B49" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C49" t="str">
-        <v>Soldadura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
+        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
       </c>
       <c r="B50" t="str">
-        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C50" t="str">
         <v>Riesgo Eléctrico</v>
@@ -967,98 +967,98 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RECICLAJE  ALTURAS TELCO I</v>
       </c>
       <c r="B51" t="str">
-        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C51" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
+        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="B52" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
       </c>
       <c r="C52" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
+        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B53" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C53" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>RIESGO ELÉCTRICO TELCO</v>
+        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B54" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C54" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
+        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="B55" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C55" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>FORMACIÓN PREVENTIVA DE RECICLAJE PARA OPERARIOS EN TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR SEGÚN UNE 171370-1</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B56" t="str">
-        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C56" t="str">
-        <v>Amianto</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
+        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B57" t="str">
-        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C57" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B58" t="str">
-        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C58" t="str">
-        <v>Construcción</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B59" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C59" t="str">
         <v>Metal</v>
@@ -1066,10 +1066,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B60" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C60" t="str">
         <v>Metal</v>
@@ -1077,10 +1077,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B61" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C61" t="str">
         <v>Metal</v>
@@ -1088,21 +1088,21 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>Mantenimiento de maquinaria y vehículos  en obras de construcción</v>
       </c>
       <c r="B62" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="C62" t="str">
-        <v>Metal</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Mantenimiento de maquinaria y vehículos  en obras de construcción</v>
+        <v>Mantenimiento de maquinaria y vehículos en obras de construcción</v>
       </c>
       <c r="B63" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C63" t="str">
         <v>Construcción</v>
@@ -1110,95 +1110,95 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
       </c>
       <c r="B64" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
       </c>
       <c r="C64" t="str">
-        <v>Metal</v>
+        <v>Incendios</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>OTROS OFICIOS DEL METAL</v>
+        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B65" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
       </c>
       <c r="C65" t="str">
-        <v>Metal</v>
+        <v>Incendios</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>ACOSO LABORAL Y SEXUAL</v>
       </c>
       <c r="B66" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="C66" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>ADMINISTRATIVOS</v>
       </c>
       <c r="B67" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C67" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
+        <v>ALBAÑILERÍA</v>
       </c>
       <c r="B68" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v/>
       </c>
       <c r="C68" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Mantenimiento de maquinaria y vehículos en obras de construcción</v>
+        <v>Campaña Allive 80.0 Fase II-Técnico de Prevención por un día-EL ALTO</v>
       </c>
       <c r="B69" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>Construcción</v>
+        <v>—</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>OPERARIOS DE INSTALACIÓN Y MANTENIMIENTO DE EQUIPOS CONTRA INCENDIOS</v>
+        <v>CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B70" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v/>
       </c>
       <c r="C70" t="str">
-        <v>Incendios</v>
+        <v>—</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
+        <v>CONDUCCIÓN SEGURA</v>
       </c>
       <c r="B71" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v/>
       </c>
       <c r="C71" t="str">
-        <v>Incendios</v>
+        <v>Conducción</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>ACOSO LABORAL Y SEXUAL</v>
+        <v>CONDUCTORES Y TRANSPORTISTAS</v>
       </c>
       <c r="B72" t="str">
         <v/>
@@ -1209,7 +1209,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>ADMINISTRATIVOS</v>
+        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="B73" t="str">
         <v/>
@@ -1220,7 +1220,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>ALBAÑILERÍA</v>
+        <v>CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="B74" t="str">
         <v/>
@@ -1231,18 +1231,18 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Campaña Allive 80.0 Fase II-Técnico de Prevención por un día-EL ALTO</v>
+        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
       </c>
       <c r="B75" t="str">
         <v/>
       </c>
       <c r="C75" t="str">
-        <v>—</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>CARPINTERÍA METÁLICA</v>
+        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="B76" t="str">
         <v/>
@@ -1253,18 +1253,18 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>CONDUCCIÓN SEGURA</v>
+        <v>ENCOFRADOS</v>
       </c>
       <c r="B77" t="str">
         <v/>
       </c>
       <c r="C77" t="str">
-        <v>Conducción</v>
+        <v>—</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>CONDUCTORES Y TRANSPORTISTAS</v>
+        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
       </c>
       <c r="B78" t="str">
         <v/>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>ESTABILIZACIÓN DE EXPLANADAS Y EXTENDIDO DE FIRMES</v>
       </c>
       <c r="B79" t="str">
         <v/>
@@ -1286,10 +1286,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v/>
       </c>
       <c r="B80" t="str">
-        <v/>
+        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
       </c>
       <c r="C80" t="str">
         <v>—</v>
@@ -1297,18 +1297,18 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
+        <v>FERRALLADO</v>
       </c>
       <c r="B81" t="str">
         <v/>
       </c>
       <c r="C81" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B82" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>ENCOFRADOS</v>
+        <v>FORMACIÓN DE INTERVENCIÓN EN EQUIPOS Y MÁQUINAS</v>
       </c>
       <c r="B83" t="str">
         <v/>
@@ -1330,7 +1330,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
+        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
       </c>
       <c r="B84" t="str">
         <v/>
@@ -1341,51 +1341,51 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>ESTABILIZACIÓN DE EXPLANADAS Y EXTENDIDO DE FIRMES</v>
+        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
       </c>
       <c r="B85" t="str">
         <v/>
       </c>
       <c r="C85" t="str">
-        <v>—</v>
+        <v>Grúa, Seguridad</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v/>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
       </c>
       <c r="B86" t="str">
-        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
+        <v/>
       </c>
       <c r="C86" t="str">
-        <v>—</v>
+        <v>PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>FERRALLADO</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
       </c>
       <c r="B87" t="str">
         <v/>
       </c>
       <c r="C87" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
       </c>
       <c r="B88" t="str">
         <v/>
       </c>
       <c r="C88" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>FORMACIÓN TEÓRICA SOBRE LA IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
       </c>
       <c r="B89" t="str">
         <v/>
@@ -1396,10 +1396,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>FORMACIÓN DE INTERVENCIÓN EN EQUIPOS Y MÁQUINAS</v>
+        <v/>
       </c>
       <c r="B90" t="str">
-        <v/>
+        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C90" t="str">
         <v>—</v>
@@ -1407,7 +1407,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
+        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
       </c>
       <c r="B91" t="str">
         <v/>
@@ -1418,76 +1418,76 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
+        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
       </c>
       <c r="B92" t="str">
         <v/>
       </c>
       <c r="C92" t="str">
-        <v>Grúa, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
+        <v/>
       </c>
       <c r="B93" t="str">
-        <v/>
+        <v>INFECCIONES RESPIRATORIAS AGUDAS</v>
       </c>
       <c r="C93" t="str">
-        <v>PRL, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B94" t="str">
         <v/>
       </c>
       <c r="C94" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
       </c>
       <c r="B95" t="str">
         <v/>
       </c>
       <c r="C95" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>FORMACIÓN TEÓRICA SOBRE LA IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
+        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
       </c>
       <c r="B96" t="str">
         <v/>
       </c>
       <c r="C96" t="str">
-        <v>—</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>FORMACIÓN TEÓRICO-PRÁCTICA SOBRE IMPLANTACION DEL PLAN EMERGENCIA. SIMULACRO DE EVACUACION</v>
+        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
       </c>
       <c r="B97" t="str">
         <v/>
       </c>
       <c r="C97" t="str">
-        <v>Emergencias</v>
+        <v>—</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v/>
+        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B98" t="str">
-        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C98" t="str">
         <v>—</v>
@@ -1495,7 +1495,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
+        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
       </c>
       <c r="B99" t="str">
         <v/>
@@ -1506,7 +1506,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
+        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B100" t="str">
         <v/>
@@ -1517,10 +1517,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v/>
+        <v>MANIPULACION DE ALIMENTOS</v>
       </c>
       <c r="B101" t="str">
-        <v>INFECCIONES RESPIRATORIAS AGUDAS</v>
+        <v/>
       </c>
       <c r="C101" t="str">
         <v>—</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v/>
       </c>
       <c r="B102" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS</v>
       </c>
       <c r="C102" t="str">
         <v>—</v>
@@ -1539,10 +1539,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="B103" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
       </c>
       <c r="C103" t="str">
         <v>—</v>
@@ -1550,7 +1550,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
+        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B104" t="str">
         <v/>
@@ -1561,7 +1561,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B105" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
+        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B106" t="str">
         <v/>
@@ -1583,18 +1583,18 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>MEDIDAS DE EMERGENCIA</v>
       </c>
       <c r="B107" t="str">
         <v/>
       </c>
       <c r="C107" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>MANIPULACION DE ALIMENTOS</v>
+        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="B108" t="str">
         <v/>
@@ -1605,10 +1605,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v/>
+        <v>MONTAJE ANDAMIOS APOYADOS</v>
       </c>
       <c r="B109" t="str">
-        <v>MANIPULADOR DE ALIMENTOS</v>
+        <v/>
       </c>
       <c r="C109" t="str">
         <v>—</v>
@@ -1616,10 +1616,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v/>
+        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
       </c>
       <c r="B110" t="str">
-        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
+        <v/>
       </c>
       <c r="C110" t="str">
         <v>—</v>
@@ -1627,10 +1627,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v/>
       </c>
       <c r="B111" t="str">
-        <v/>
+        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C111" t="str">
         <v>—</v>
@@ -1638,7 +1638,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
+        <v>OPERACIONES TELCO</v>
       </c>
       <c r="B112" t="str">
         <v/>
@@ -1649,29 +1649,29 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>OPERADOR DE CAMIÓN GRÚA</v>
       </c>
       <c r="B113" t="str">
         <v/>
       </c>
       <c r="C113" t="str">
-        <v>—</v>
+        <v>Grúa</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>MEDIDAS DE EMERGENCIA</v>
+        <v>OPERADOR DE PALA CARGADORA</v>
       </c>
       <c r="B114" t="str">
         <v/>
       </c>
       <c r="C114" t="str">
-        <v>Emergencias</v>
+        <v>—</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B115" t="str">
         <v/>
@@ -1682,18 +1682,18 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>MONTAJE ANDAMIOS APOYADOS</v>
+        <v>OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="B116" t="str">
         <v/>
       </c>
       <c r="C116" t="str">
-        <v>—</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
+        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B117" t="str">
         <v/>
@@ -1704,10 +1704,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v/>
+        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B118" t="str">
-        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C118" t="str">
         <v>—</v>
@@ -1715,18 +1715,18 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>NIVEL BÁSICO EN PREVENCIÓN DE RIESGOS LABORALES 50 H</v>
+        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
       </c>
       <c r="B119" t="str">
         <v/>
       </c>
       <c r="C119" t="str">
-        <v>PRL, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>OPERACIONES TELCO</v>
+        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
       </c>
       <c r="B120" t="str">
         <v/>
@@ -1737,18 +1737,18 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>OPERADOR DE CAMIÓN GRÚA</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B121" t="str">
         <v/>
       </c>
       <c r="C121" t="str">
-        <v>Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>OPERADOR DE PALA CARGADORA</v>
+        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B122" t="str">
         <v/>
@@ -1759,7 +1759,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>OPERADORES DE APARATOS ELEVADORES</v>
+        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B123" t="str">
         <v/>
@@ -1770,18 +1770,18 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>OPERADORES DE PUENTE-GRÚA</v>
+        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
       </c>
       <c r="B124" t="str">
         <v/>
       </c>
       <c r="C124" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>OTRO TIPO DE INSTALACIONES</v>
       </c>
       <c r="B125" t="str">
         <v/>
@@ -1792,7 +1792,7 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>PINTURA</v>
       </c>
       <c r="B126" t="str">
         <v/>
@@ -1803,29 +1803,29 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
+        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
       </c>
       <c r="B127" t="str">
         <v/>
       </c>
       <c r="C127" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
       </c>
       <c r="B128" t="str">
         <v/>
       </c>
       <c r="C128" t="str">
-        <v>—</v>
+        <v>PEMP, Seguridad</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
       </c>
       <c r="B129" t="str">
         <v/>
@@ -1836,117 +1836,117 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
       </c>
       <c r="B130" t="str">
         <v/>
       </c>
       <c r="C130" t="str">
-        <v>—</v>
+        <v>Ergonomía, PRL</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
       </c>
       <c r="B131" t="str">
         <v/>
       </c>
       <c r="C131" t="str">
-        <v>—</v>
+        <v>Grúa, PRL</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B132" t="str">
         <v/>
       </c>
       <c r="C132" t="str">
-        <v>—</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>OTRO TIPO DE INSTALACIONES</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
       </c>
       <c r="B133" t="str">
         <v/>
       </c>
       <c r="C133" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>PINTURA</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
       </c>
       <c r="B134" t="str">
         <v/>
       </c>
       <c r="C134" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
+        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
       </c>
       <c r="B135" t="str">
         <v/>
       </c>
       <c r="C135" t="str">
-        <v>Emergencias</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
+        <v/>
       </c>
       <c r="B136" t="str">
-        <v/>
+        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C136" t="str">
-        <v>PEMP, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
+        <v>Primeros Auxilios en Equipos de Emergencia</v>
       </c>
       <c r="B137" t="str">
         <v/>
       </c>
       <c r="C137" t="str">
-        <v>—</v>
+        <v>Primeros Auxilios, Emergencias</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
+        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
       </c>
       <c r="B138" t="str">
         <v/>
       </c>
       <c r="C138" t="str">
-        <v>Ergonomía, PRL</v>
+        <v>Primeros Auxilios, Emergencias</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
+        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
       </c>
       <c r="B139" t="str">
         <v/>
       </c>
       <c r="C139" t="str">
-        <v>Grúa, PRL</v>
+        <v>Manipulación Cargas, PRL</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
+        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B140" t="str">
         <v/>
@@ -1957,35 +1957,35 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
+        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B141" t="str">
         <v/>
       </c>
       <c r="C141" t="str">
-        <v>PRL</v>
+        <v>PEMP, Plataformas, PRL</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
+        <v/>
       </c>
       <c r="B142" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C142" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
+        <v/>
       </c>
       <c r="B143" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C143" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="144">
@@ -1993,65 +1993,65 @@
         <v/>
       </c>
       <c r="B144" t="str">
-        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C144" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>Primeros Auxilios en Equipos de Emergencia</v>
+        <v/>
       </c>
       <c r="B145" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C145" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
+        <v/>
       </c>
       <c r="B146" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C146" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
+        <v/>
       </c>
       <c r="B147" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C147" t="str">
-        <v>Manipulación Cargas, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B148" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C148" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B149" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C149" t="str">
-        <v>PEMP, Plataformas, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="150">
@@ -2059,7 +2059,7 @@
         <v/>
       </c>
       <c r="B150" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C150" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2070,7 +2070,7 @@
         <v/>
       </c>
       <c r="B151" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C151" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2081,7 +2081,7 @@
         <v/>
       </c>
       <c r="B152" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C152" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="B153" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C153" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2103,7 +2103,7 @@
         <v/>
       </c>
       <c r="B154" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C154" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="B155" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C155" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2125,7 +2125,7 @@
         <v/>
       </c>
       <c r="B156" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C156" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2136,7 +2136,7 @@
         <v/>
       </c>
       <c r="B157" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C157" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2144,57 +2144,57 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v/>
+        <v>PRL SEGURIDAD VIAL</v>
       </c>
       <c r="B158" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v/>
       </c>
       <c r="C158" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL, Seguridad</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v/>
+        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
       </c>
       <c r="B159" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v/>
       </c>
       <c r="C159" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v/>
+        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
       </c>
       <c r="B160" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v/>
       </c>
       <c r="C160" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v/>
+        <v>PRODQUIM/000</v>
       </c>
       <c r="B161" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="C161" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v/>
+        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B162" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C162" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="163">
@@ -2202,10 +2202,10 @@
         <v/>
       </c>
       <c r="B163" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C163" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="164">
@@ -2213,10 +2213,10 @@
         <v/>
       </c>
       <c r="B164" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C164" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="165">
@@ -2224,59 +2224,59 @@
         <v/>
       </c>
       <c r="B165" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C165" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>PRL SEGURIDAD VIAL</v>
+        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B166" t="str">
         <v/>
       </c>
       <c r="C166" t="str">
-        <v>PRL, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
+        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B167" t="str">
         <v/>
       </c>
       <c r="C167" t="str">
-        <v>PRL</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
+        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B168" t="str">
         <v/>
       </c>
       <c r="C168" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>PRODQUIM/000</v>
+        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B169" t="str">
         <v/>
       </c>
       <c r="C169" t="str">
-        <v>—</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>RECICLAJE PARA FERRALLADO</v>
       </c>
       <c r="B170" t="str">
         <v/>
@@ -2287,62 +2287,62 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v/>
+        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B171" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C171" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v/>
+        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B172" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C172" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v/>
+        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B173" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C173" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B174" t="str">
         <v/>
       </c>
       <c r="C174" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
+        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B175" t="str">
         <v/>
       </c>
       <c r="C175" t="str">
-        <v>Espacios Confinados</v>
+        <v>—</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B176" t="str">
         <v/>
@@ -2353,18 +2353,18 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>RECICLAJE PARA OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="B177" t="str">
         <v/>
       </c>
       <c r="C177" t="str">
-        <v>Carretillas</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>RECICLAJE PARA FERRALLADO</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B178" t="str">
         <v/>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B179" t="str">
         <v/>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B180" t="str">
         <v/>
@@ -2397,7 +2397,7 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
       </c>
       <c r="B181" t="str">
         <v/>
@@ -2408,7 +2408,7 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B182" t="str">
         <v/>
@@ -2419,95 +2419,95 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v/>
       </c>
       <c r="B183" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C183" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="B184" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C184" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>RECICLAJE PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B185" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C185" t="str">
-        <v>PEMP, Plataformas</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>RECICLAJE PARA OPERADORES DE PUENTE-GRÚA</v>
+        <v/>
       </c>
       <c r="B186" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C21- TRABAJOS DE INSTALACIONES, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES (TIC Y DIGITALIZACIÓN)</v>
       </c>
       <c r="C186" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="B187" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C23- TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C187" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="B188" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C188" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="B189" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C189" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v/>
       </c>
       <c r="B190" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C190" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
       </c>
       <c r="B191" t="str">
         <v/>
@@ -2518,46 +2518,46 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v/>
+        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B192" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C192" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v/>
+        <v>REVESTIMIENTO DE YESO</v>
       </c>
       <c r="B193" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v/>
       </c>
       <c r="C193" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v/>
+        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
       </c>
       <c r="B194" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="C194" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v/>
+        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
       </c>
       <c r="B195" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C195" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="196">
@@ -2565,10 +2565,10 @@
         <v/>
       </c>
       <c r="B196" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C196" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="197">
@@ -2576,65 +2576,65 @@
         <v/>
       </c>
       <c r="B197" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C197" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
+        <v/>
       </c>
       <c r="B198" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C198" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v/>
       </c>
       <c r="B199" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C199" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>REVESTIMIENTO DE YESO</v>
+        <v/>
       </c>
       <c r="B200" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="C200" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
+        <v/>
       </c>
       <c r="B201" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C201" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
+        <v/>
       </c>
       <c r="B202" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C202" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="203">
@@ -2642,7 +2642,7 @@
         <v/>
       </c>
       <c r="B203" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20  HORAS): CIMENTACIONES ESPECIALES, SONDEOS Y PERFORACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
       </c>
       <c r="C203" t="str">
         <v>Construcción, PRL</v>
@@ -2653,7 +2653,7 @@
         <v/>
       </c>
       <c r="B204" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C204" t="str">
         <v>Construcción, PRL</v>
@@ -2664,7 +2664,7 @@
         <v/>
       </c>
       <c r="B205" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C205" t="str">
         <v>Construcción, PRL</v>
@@ -2675,7 +2675,7 @@
         <v/>
       </c>
       <c r="B206" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C206" t="str">
         <v>Construcción, PRL</v>
@@ -2686,7 +2686,7 @@
         <v/>
       </c>
       <c r="B207" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C207" t="str">
         <v>Construcción, PRL</v>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="B208" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C208" t="str">
         <v>Construcción, PRL</v>
@@ -2708,7 +2708,7 @@
         <v/>
       </c>
       <c r="B209" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGON EN OBRA</v>
       </c>
       <c r="C209" t="str">
         <v>Construcción, PRL</v>
@@ -2719,7 +2719,7 @@
         <v/>
       </c>
       <c r="B210" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C210" t="str">
         <v>Construcción, PRL</v>
@@ -2730,7 +2730,7 @@
         <v/>
       </c>
       <c r="B211" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C211" t="str">
         <v>Construcción, PRL</v>
@@ -2741,7 +2741,7 @@
         <v/>
       </c>
       <c r="B212" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CIMENTACIONES ESPECIALES, SONDEOS Y PERFORACIONES</v>
       </c>
       <c r="C212" t="str">
         <v>Construcción, PRL</v>
@@ -2752,7 +2752,7 @@
         <v/>
       </c>
       <c r="B213" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C213" t="str">
         <v>Construcción, PRL</v>
@@ -2763,7 +2763,7 @@
         <v/>
       </c>
       <c r="B214" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C214" t="str">
         <v>Construcción, PRL</v>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="B215" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="C215" t="str">
         <v>Construcción, PRL</v>
@@ -2785,7 +2785,7 @@
         <v/>
       </c>
       <c r="B216" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C216" t="str">
         <v>Construcción, PRL</v>
@@ -2796,7 +2796,7 @@
         <v/>
       </c>
       <c r="B217" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C217" t="str">
         <v>Construcción, PRL</v>
@@ -2807,7 +2807,7 @@
         <v/>
       </c>
       <c r="B218" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
       </c>
       <c r="C218" t="str">
         <v>Construcción, PRL</v>
@@ -2818,7 +2818,7 @@
         <v/>
       </c>
       <c r="B219" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C219" t="str">
         <v>Construcción, PRL</v>
@@ -2829,7 +2829,7 @@
         <v/>
       </c>
       <c r="B220" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CIMENTACIONES ESPECIALES, SONDEOS Y PERFORACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C220" t="str">
         <v>Construcción, PRL</v>
@@ -2840,7 +2840,7 @@
         <v/>
       </c>
       <c r="B221" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C221" t="str">
         <v>Construcción, PRL</v>
@@ -2851,7 +2851,7 @@
         <v/>
       </c>
       <c r="B222" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C222" t="str">
         <v>Construcción, PRL</v>
@@ -2862,7 +2862,7 @@
         <v/>
       </c>
       <c r="B223" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C223" t="str">
         <v>Construcción, PRL</v>
@@ -2873,7 +2873,7 @@
         <v/>
       </c>
       <c r="B224" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGON EN OBRA</v>
       </c>
       <c r="C224" t="str">
         <v>Construcción, PRL</v>
@@ -2884,10 +2884,10 @@
         <v/>
       </c>
       <c r="B225" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C225" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="226">
@@ -2895,10 +2895,10 @@
         <v/>
       </c>
       <c r="B226" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C226" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="227">
@@ -2906,10 +2906,10 @@
         <v/>
       </c>
       <c r="B227" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C227" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="228">
@@ -2917,10 +2917,10 @@
         <v/>
       </c>
       <c r="B228" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C228" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="229">
@@ -2928,10 +2928,10 @@
         <v/>
       </c>
       <c r="B229" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C229" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="230">
@@ -2939,10 +2939,10 @@
         <v/>
       </c>
       <c r="B230" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C230" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="231">
@@ -2950,10 +2950,10 @@
         <v/>
       </c>
       <c r="B231" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C231" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="232">
@@ -2961,10 +2961,10 @@
         <v/>
       </c>
       <c r="B232" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C232" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="233">
@@ -2972,7 +2972,7 @@
         <v/>
       </c>
       <c r="B233" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C233" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2983,7 +2983,7 @@
         <v/>
       </c>
       <c r="B234" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): MANDOS INTERMEDIOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C234" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2994,7 +2994,7 @@
         <v/>
       </c>
       <c r="B235" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C235" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3005,7 +3005,7 @@
         <v/>
       </c>
       <c r="B236" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C236" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -3013,304 +3013,304 @@
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v/>
+        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
       </c>
       <c r="B237" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C237" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
       </c>
       <c r="B238" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C238" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
       </c>
       <c r="B239" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C239" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
       </c>
       <c r="B240" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C240" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
       </c>
       <c r="B241" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C241" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA. RECICLAJE</v>
       </c>
       <c r="B242" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v/>
       </c>
       <c r="C242" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Puente Grúa, Grúa, Seguridad</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B243" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C243" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
       </c>
       <c r="B244" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C244" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v/>
+        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B245" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C245" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B246" t="str">
         <v/>
       </c>
       <c r="C246" t="str">
-        <v>Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
       </c>
       <c r="B247" t="str">
         <v/>
       </c>
       <c r="C247" t="str">
-        <v>Seguridad</v>
+        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
       </c>
       <c r="B248" t="str">
         <v/>
       </c>
       <c r="C248" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
       </c>
       <c r="B249" t="str">
         <v/>
       </c>
       <c r="C249" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
       </c>
       <c r="B250" t="str">
         <v/>
       </c>
       <c r="C250" t="str">
-        <v>Seguridad</v>
+        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA. RECICLAJE</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
       </c>
       <c r="B251" t="str">
         <v/>
       </c>
       <c r="C251" t="str">
-        <v>Puente Grúa, Grúa, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
       </c>
       <c r="B252" t="str">
         <v/>
       </c>
       <c r="C252" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
+        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
       </c>
       <c r="B253" t="str">
         <v/>
       </c>
       <c r="C253" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>Riesgo Químico, Seguridad</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
       </c>
       <c r="B254" t="str">
         <v/>
       </c>
       <c r="C254" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
+        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
       </c>
       <c r="B255" t="str">
         <v/>
       </c>
       <c r="C255" t="str">
-        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
+        <v>Grúa, Conducción Vehículos</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
+        <v>SOLADOS Y ALICATADOS</v>
       </c>
       <c r="B256" t="str">
         <v/>
       </c>
       <c r="C256" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B257" t="str">
         <v/>
       </c>
       <c r="C257" t="str">
-        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B258" t="str">
         <v/>
       </c>
       <c r="C258" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
+        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B259" t="str">
         <v/>
       </c>
       <c r="C259" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
+        <v/>
       </c>
       <c r="B260" t="str">
-        <v/>
+        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C260" t="str">
-        <v>Riesgo Químico, Seguridad</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE TRANSPALETAS ELÉCTRICAS Y TRANSPALETAS MANUALES</v>
+        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
       </c>
       <c r="B261" t="str">
         <v/>
       </c>
       <c r="C261" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
+        <v>TRABAJOS DE ARQUEOLOGÍA</v>
       </c>
       <c r="B262" t="str">
         <v/>
       </c>
       <c r="C262" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
+        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B263" t="str">
         <v/>
       </c>
       <c r="C263" t="str">
-        <v>Grúa, Conducción Vehículos</v>
+        <v>—</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>SOLADOS Y ALICATADOS</v>
+        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
       </c>
       <c r="B264" t="str">
         <v/>
@@ -3321,40 +3321,40 @@
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
       </c>
       <c r="B265" t="str">
         <v/>
       </c>
       <c r="C265" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v>TRABAJOS DE SOLDADURA</v>
       </c>
       <c r="B266" t="str">
         <v/>
       </c>
       <c r="C266" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
       </c>
       <c r="B267" t="str">
         <v/>
       </c>
       <c r="C267" t="str">
-        <v>—</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>TEÓRICO-PRÁCTICO DE MONTAJE DE PUNTOS DE ANCLAJE Y LÍNEAS DE VIDA PROVISIONALES</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
       </c>
       <c r="B268" t="str">
         <v/>
@@ -3365,106 +3365,18 @@
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
       </c>
       <c r="B269" t="str">
         <v/>
       </c>
       <c r="C269" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="str">
-        <v>TRABAJOS DE ARQUEOLOGÍA</v>
-      </c>
-      <c r="B270" t="str">
-        <v/>
-      </c>
-      <c r="C270" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="str">
-        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
-      </c>
-      <c r="B271" t="str">
-        <v/>
-      </c>
-      <c r="C271" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="str">
-        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
-      </c>
-      <c r="B272" t="str">
-        <v/>
-      </c>
-      <c r="C272" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="str">
-        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
-      </c>
-      <c r="B273" t="str">
-        <v/>
-      </c>
-      <c r="C273" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="str">
-        <v>TRABAJOS DE SOLDADURA</v>
-      </c>
-      <c r="B274" t="str">
-        <v/>
-      </c>
-      <c r="C274" t="str">
-        <v>Soldadura</v>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="str">
-        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
-      </c>
-      <c r="B275" t="str">
-        <v/>
-      </c>
-      <c r="C275" t="str">
-        <v>Trabajos en Altura</v>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
-      </c>
-      <c r="B276" t="str">
-        <v/>
-      </c>
-      <c r="C276" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
-      </c>
-      <c r="B277" t="str">
-        <v/>
-      </c>
-      <c r="C277" t="str">
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C277"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C269"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: Actualización de datos Excel y diccionario de sinergias
</commit_message>
<xml_diff>
--- a/public/data/diccionario_sinergias_final.xlsx
+++ b/public/data/diccionario_sinergias_final.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C269"/>
+  <dimension ref="A1:C265"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -428,98 +428,98 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Construcción, reparación y mantenimiento naval en astilleros y muelles</v>
+        <v>PRL PARA OPERADOR/A DEL APILADOR ELÉCTRICO</v>
       </c>
       <c r="B2" t="str">
-        <v>NIVEL BASICO DE PREVENCION DE LAS ACTIVIDADES DEL METAL EN LA CONSTRUCCION</v>
+        <v>CARRETILLAS ELEVADORAS (FRONTALES, RETRÁCTILES, TRANSPALETAS Y APILADORES ELÉCTRICOS). TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C2" t="str">
-        <v>Sector Metal, Construcción, Metal, Nivel Básico</v>
+        <v>Carretillas, Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>PRL PARA OPERADOR/A DEL APILADOR ELÉCTRICO</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Instaladores y reparadores de líneas y equipos eléctricos</v>
       </c>
       <c r="B3" t="str">
-        <v>CARRETILLAS ELEVADORAS (FRONTALES, RETRÁCTILES, TRANSPALETAS Y APILADORES ELÉCTRICOS). TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C3" t="str">
-        <v>Carretillas, Riesgo Eléctrico</v>
+        <v>Riesgo Eléctrico, Metal, PRL</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Instaladores y reparadores de líneas y equipos eléctricos</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en trabajos de soldadura y oxicorte</v>
       </c>
       <c r="B4" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C4" t="str">
-        <v>Riesgo Eléctrico, Metal, PRL</v>
+        <v>Soldadura, Metal, PRL</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en trabajos de soldadura y oxicorte</v>
+        <v>SEGURIDAD EN EL USO DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B5" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>SEGURIDAD EN EL MANEJO DE PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C5" t="str">
-        <v>Soldadura, Metal, PRL</v>
+        <v>PEMP, Plataformas, Seguridad</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SEGURIDAD EN EL USO DE PLATAFORMAS ELEVADORAS</v>
+        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA</v>
       </c>
       <c r="B6" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE PUENTES-GRÚA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C6" t="str">
-        <v>PEMP, Plataformas, Seguridad</v>
+        <v>Puente Grúa, Grúa, Seguridad</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SEGURIDAD EN EL MANEJO DEL PUENTE GRÚA</v>
+        <v>OPERADOR DE PLATAFORMAS ELEVADORAS SEGÚN UNE-58923</v>
       </c>
       <c r="B7" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE PUENTES-GRÚA. TEÓRICO-PRÁCTICO</v>
+        <v>CONDUCCION Y MANEJO SEGURO DE PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C7" t="str">
-        <v>Puente Grúa, Grúa, Seguridad</v>
+        <v>PEMP, Plataformas</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA</v>
+        <v>EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B8" t="str">
-        <v>SEGURIDAD EN EL MANEJO PUENTES-GRÚA. TEÓRICO-PRÁCTICO</v>
+        <v>EXTINCIÓN DE INCENDIOS CON INTERVENCIÓN Y EVACUACIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C8" t="str">
-        <v>Puente Grúa, Grúa, Seguridad</v>
+        <v>Extinción Incendios, Incendios</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SEGURIDAD EN EL USO DE PLATAFORMAS ELEVADORAS. RECICLAJE</v>
+        <v>EXTINCIÓN DE INCENDIOS Y PRIMEROS AUXILIOS</v>
       </c>
       <c r="B9" t="str">
-        <v>SEGURIDAD Y MANEJO CON PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>EXTINCIÓN DE INCENDIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C9" t="str">
-        <v>PEMP, Plataformas, Seguridad</v>
+        <v>Extinción Incendios, Incendios</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>OPERADOR DE PLATAFORMAS ELEVADORAS SEGÚN UNE-58923</v>
+        <v>OPERADORES DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B10" t="str">
-        <v>CONDUCCION Y MANEJO SEGURO DE PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>MANEJO SEGURO DE PLATAFORMAS ELEVADORAS SEGÚN NORMA UNE 58923:2020. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C10" t="str">
         <v>PEMP, Plataformas</v>
@@ -527,10 +527,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EXTINCIÓN DE INCENDIOS</v>
+        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
       </c>
       <c r="B11" t="str">
-        <v>EXTINCIÓN DE INCENDIOS CON INTERVENCIÓN Y EVACUACIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>PREVENCIÓN Y EXTINCIÓN DE INCENDIOS PARA EQUIPOS DE PRIMERA INTERVENCIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C11" t="str">
         <v>Extinción Incendios, Incendios</v>
@@ -538,76 +538,76 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>EXTINCIÓN DE INCENDIOS Y PRIMEROS AUXILIOS</v>
+        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
       </c>
       <c r="B12" t="str">
-        <v>EXTINCIÓN DE INCENDIOS. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="C12" t="str">
-        <v>Extinción Incendios, Incendios</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
       </c>
       <c r="B13" t="str">
-        <v>MANEJO SEGURO DE PLATAFORMAS ELEVADORAS SEGÚN NORMA UNE 58923:2020. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO PUENTES-GRÚA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C13" t="str">
-        <v>PEMP, Plataformas</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
       </c>
       <c r="B14" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>NIVEL BÁSICO PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA</v>
       </c>
       <c r="C14" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Metal, PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
+        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B15" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C15" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Carretillas, PRL</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B16" t="str">
-        <v>NIVEL BÁSICO PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA</v>
+        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C16" t="str">
-        <v>Metal, PRL, Nivel Básico</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
       </c>
       <c r="B17" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C17" t="str">
-        <v>Carretillas, PRL</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B18" t="str">
-        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C18" t="str">
         <v>Carretillas, Seguridad</v>
@@ -615,76 +615,76 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B19" t="str">
-        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C19" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B20" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C20" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
       </c>
       <c r="B21" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C21" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>ALTURAS TELCO I</v>
       </c>
       <c r="B22" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C22" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
       </c>
       <c r="B23" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>ALTURAS TELCO II. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C23" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ALTURAS TELCO I</v>
+        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B24" t="str">
-        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
+        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C24" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
       </c>
       <c r="B25" t="str">
-        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
+        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
       </c>
       <c r="C25" t="str">
         <v>Carretillas</v>
@@ -692,32 +692,32 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="B26" t="str">
-        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
+        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="C26" t="str">
-        <v>Carretillas</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B27" t="str">
-        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>ESPACIOS CONFINADOS TELCO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C27" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ESPACIOS CONFINADOS TELCO</v>
+        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
       </c>
       <c r="B28" t="str">
-        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C28" t="str">
         <v>Espacios Confinados</v>
@@ -725,186 +725,186 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
+        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B29" t="str">
-        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
+        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C29" t="str">
-        <v>Construcción, Nivel Básico</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
+        <v>PRIMEROS AUXILIOS</v>
       </c>
       <c r="B30" t="str">
-        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
+        <v>FORMACION AELEC EN PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C30" t="str">
-        <v>Metal, Nivel Básico</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
+        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
       </c>
       <c r="B31" t="str">
-        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
+        <v>NIVEL BASICO DE PREVENCION DE LAS ACTIVIDADES DEL METAL EN LA CONSTRUCCION</v>
       </c>
       <c r="C31" t="str">
-        <v>Carretillas</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PRIMEROS AUXILIOS</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
       </c>
       <c r="B32" t="str">
-        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
+        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
       </c>
       <c r="C32" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Metal, Nivel Básico</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
+        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B33" t="str">
-        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C33" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
+        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
       </c>
       <c r="B34" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C34" t="str">
-        <v>Metal, PRL</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
+        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
       </c>
       <c r="B35" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C35" t="str">
-        <v>Metal, PRL</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B36" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C36" t="str">
-        <v>Metal, PRL</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
+        <v>RECICLAJE  ALTURAS TELCO I</v>
       </c>
       <c r="B37" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>PRL EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C37" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
+        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
       </c>
       <c r="B38" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C38" t="str">
-        <v>Carretillas</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
       </c>
       <c r="B39" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C39" t="str">
-        <v>Soldadura</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
       </c>
       <c r="B40" t="str">
-        <v>RECICLAJE ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C40" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
+        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
       </c>
       <c r="B41" t="str">
-        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C41" t="str">
-        <v>Amianto</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
       </c>
       <c r="B42" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C42" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
+        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B43" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C15- INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C43" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
       </c>
       <c r="B44" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
       </c>
       <c r="C44" t="str">
-        <v>Soldadura</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
+        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B45" t="str">
-        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C45" t="str">
         <v>Riesgo Eléctrico</v>
@@ -912,21 +912,21 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B46" t="str">
-        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C46" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
+        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
       </c>
       <c r="B47" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>RIESGO ELÉCTRICO . TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C47" t="str">
         <v>Riesgo Eléctrico</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
+        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
       </c>
       <c r="B48" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C48" t="str">
         <v>Riesgo Eléctrico</v>
@@ -945,10 +945,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RIESGO ELÉCTRICO TELCO</v>
+        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B49" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C49" t="str">
         <v>Riesgo Eléctrico</v>
@@ -956,10 +956,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
+        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B50" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C50" t="str">
         <v>Riesgo Eléctrico</v>
@@ -967,76 +967,76 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>RECICLAJE  ALTURAS TELCO I</v>
+        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
       </c>
       <c r="B51" t="str">
-        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C51" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B52" t="str">
-        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C52" t="str">
-        <v>Construcción</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
       </c>
       <c r="B53" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C53" t="str">
-        <v>Metal</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
+        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B54" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>SEGURIDAD CONTRA INCENDIOS Y ACTUACIÓN ANTE EMERGENCIAS. TEÓRICO-PRÁCTICO.</v>
       </c>
       <c r="C54" t="str">
-        <v>Metal</v>
+        <v>Incendios, Seguridad</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
       </c>
       <c r="B55" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C55" t="str">
-        <v>Metal</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="B56" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
       </c>
       <c r="C56" t="str">
-        <v>Metal</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B57" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C57" t="str">
         <v>Metal</v>
@@ -1044,10 +1044,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>OTROS OFICIOS DEL METAL</v>
+        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B58" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C58" t="str">
         <v>Metal</v>
@@ -1055,10 +1055,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="B59" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C59" t="str">
         <v>Metal</v>
@@ -1066,10 +1066,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B60" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C60" t="str">
         <v>Metal</v>
@@ -1077,10 +1077,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
+        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B61" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C61" t="str">
         <v>Metal</v>
@@ -1088,46 +1088,46 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Mantenimiento de maquinaria y vehículos  en obras de construcción</v>
+        <v>OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B62" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
       </c>
       <c r="C62" t="str">
-        <v>Construcción</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Mantenimiento de maquinaria y vehículos en obras de construcción</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B63" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C63" t="str">
-        <v>Construcción</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B64" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C64" t="str">
-        <v>Incendios</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
+        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B65" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C65" t="str">
-        <v>Incendios</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="66">
@@ -1319,7 +1319,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>FORMACIÓN DE INTERVENCIÓN EN EQUIPOS Y MÁQUINAS</v>
+        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
       </c>
       <c r="B83" t="str">
         <v/>
@@ -1330,40 +1330,40 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
+        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
       </c>
       <c r="B84" t="str">
         <v/>
       </c>
       <c r="C84" t="str">
-        <v>—</v>
+        <v>Grúa, Seguridad</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
       </c>
       <c r="B85" t="str">
         <v/>
       </c>
       <c r="C85" t="str">
-        <v>Grúa, Seguridad</v>
+        <v>PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
       </c>
       <c r="B86" t="str">
         <v/>
       </c>
       <c r="C86" t="str">
-        <v>PRL, Nivel Básico</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
       </c>
       <c r="B87" t="str">
         <v/>
@@ -1374,18 +1374,18 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
+        <v/>
       </c>
       <c r="B88" t="str">
-        <v/>
+        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C88" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>FORMACIÓN TEÓRICA SOBRE LA IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
+        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
       </c>
       <c r="B89" t="str">
         <v/>
@@ -1396,10 +1396,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v/>
+        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
       </c>
       <c r="B90" t="str">
-        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C90" t="str">
         <v>—</v>
@@ -1407,10 +1407,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
+        <v/>
       </c>
       <c r="B91" t="str">
-        <v/>
+        <v>INFECCIONES RESPIRATORIAS AGUDAS</v>
       </c>
       <c r="C91" t="str">
         <v>—</v>
@@ -1418,7 +1418,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B92" t="str">
         <v/>
@@ -1429,10 +1429,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v/>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
       </c>
       <c r="B93" t="str">
-        <v>INFECCIONES RESPIRATORIAS AGUDAS</v>
+        <v/>
       </c>
       <c r="C93" t="str">
         <v>—</v>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
       </c>
       <c r="B94" t="str">
         <v/>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
+        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B95" t="str">
         <v/>
@@ -1462,18 +1462,18 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
+        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
       </c>
       <c r="B96" t="str">
         <v/>
       </c>
       <c r="C96" t="str">
-        <v>Espacios Confinados</v>
+        <v>—</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
+        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B97" t="str">
         <v/>
@@ -1484,7 +1484,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>MANIPULACION DE ALIMENTOS</v>
       </c>
       <c r="B98" t="str">
         <v/>
@@ -1495,10 +1495,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
+        <v/>
       </c>
       <c r="B99" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS</v>
       </c>
       <c r="C99" t="str">
         <v>—</v>
@@ -1506,10 +1506,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v/>
       </c>
       <c r="B100" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
       </c>
       <c r="C100" t="str">
         <v>—</v>
@@ -1517,7 +1517,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>MANIPULACION DE ALIMENTOS</v>
+        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B101" t="str">
         <v/>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v/>
+        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B102" t="str">
-        <v>MANIPULADOR DE ALIMENTOS</v>
+        <v/>
       </c>
       <c r="C102" t="str">
         <v>—</v>
@@ -1539,10 +1539,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v/>
+        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B103" t="str">
-        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
+        <v/>
       </c>
       <c r="C103" t="str">
         <v>—</v>
@@ -1550,18 +1550,18 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>MEDIDAS DE EMERGENCIA</v>
       </c>
       <c r="B104" t="str">
         <v/>
       </c>
       <c r="C104" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
+        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="B105" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>MONTAJE ANDAMIOS APOYADOS</v>
       </c>
       <c r="B106" t="str">
         <v/>
@@ -1583,21 +1583,21 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>MEDIDAS DE EMERGENCIA</v>
+        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
       </c>
       <c r="B107" t="str">
         <v/>
       </c>
       <c r="C107" t="str">
-        <v>Emergencias</v>
+        <v>—</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v/>
       </c>
       <c r="B108" t="str">
-        <v/>
+        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C108" t="str">
         <v>—</v>
@@ -1605,7 +1605,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>MONTAJE ANDAMIOS APOYADOS</v>
+        <v>OPERACIONES TELCO</v>
       </c>
       <c r="B109" t="str">
         <v/>
@@ -1616,21 +1616,21 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
+        <v>OPERADOR DE CAMIÓN GRÚA</v>
       </c>
       <c r="B110" t="str">
         <v/>
       </c>
       <c r="C110" t="str">
-        <v>—</v>
+        <v>Grúa</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v/>
+        <v>OPERADOR DE PALA CARGADORA</v>
       </c>
       <c r="B111" t="str">
-        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C111" t="str">
         <v>—</v>
@@ -1638,7 +1638,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>OPERACIONES TELCO</v>
+        <v>OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B112" t="str">
         <v/>
@@ -1649,18 +1649,18 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>OPERADOR DE CAMIÓN GRÚA</v>
+        <v>OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="B113" t="str">
         <v/>
       </c>
       <c r="C113" t="str">
-        <v>Grúa</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>OPERADOR DE PALA CARGADORA</v>
+        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B114" t="str">
         <v/>
@@ -1671,7 +1671,7 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>OPERADORES DE APARATOS ELEVADORES</v>
+        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B115" t="str">
         <v/>
@@ -1682,29 +1682,29 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>OPERADORES DE PUENTE-GRÚA</v>
+        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
       </c>
       <c r="B116" t="str">
         <v/>
       </c>
       <c r="C116" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v/>
       </c>
       <c r="B117" t="str">
-        <v/>
+        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
       </c>
       <c r="C117" t="str">
-        <v>—</v>
+        <v>Construcción</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
       </c>
       <c r="B118" t="str">
         <v/>
@@ -1715,7 +1715,7 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B119" t="str">
         <v/>
@@ -1726,7 +1726,7 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
+        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B120" t="str">
         <v/>
@@ -1737,7 +1737,7 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B121" t="str">
         <v/>
@@ -1748,7 +1748,7 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
       </c>
       <c r="B122" t="str">
         <v/>
@@ -1759,7 +1759,7 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>OTRO TIPO DE INSTALACIONES</v>
       </c>
       <c r="B123" t="str">
         <v/>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v>PINTURA</v>
       </c>
       <c r="B124" t="str">
         <v/>
@@ -1781,95 +1781,95 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>OTRO TIPO DE INSTALACIONES</v>
+        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
       </c>
       <c r="B125" t="str">
         <v/>
       </c>
       <c r="C125" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>PINTURA</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
       </c>
       <c r="B126" t="str">
         <v/>
       </c>
       <c r="C126" t="str">
-        <v>—</v>
+        <v>PEMP, Seguridad</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
+        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
       </c>
       <c r="B127" t="str">
         <v/>
       </c>
       <c r="C127" t="str">
-        <v>Emergencias</v>
+        <v>—</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
+        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
       </c>
       <c r="B128" t="str">
         <v/>
       </c>
       <c r="C128" t="str">
-        <v>PEMP, Seguridad</v>
+        <v>Ergonomía, PRL</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
       </c>
       <c r="B129" t="str">
         <v/>
       </c>
       <c r="C129" t="str">
-        <v>—</v>
+        <v>Grúa, PRL</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
+        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B130" t="str">
         <v/>
       </c>
       <c r="C130" t="str">
-        <v>Ergonomía, PRL</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
       </c>
       <c r="B131" t="str">
         <v/>
       </c>
       <c r="C131" t="str">
-        <v>Grúa, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
       </c>
       <c r="B132" t="str">
         <v/>
       </c>
       <c r="C132" t="str">
-        <v>ATEX, PRL</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
+        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
       </c>
       <c r="B133" t="str">
         <v/>
@@ -1880,90 +1880,90 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
+        <v/>
       </c>
       <c r="B134" t="str">
-        <v/>
+        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C134" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
+        <v>Primeros Auxilios en Equipos de Emergencia</v>
       </c>
       <c r="B135" t="str">
         <v/>
       </c>
       <c r="C135" t="str">
-        <v>PRL</v>
+        <v>Primeros Auxilios, Emergencias</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v/>
+        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
       </c>
       <c r="B136" t="str">
-        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C136" t="str">
-        <v>—</v>
+        <v>Manipulación Cargas, PRL</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Primeros Auxilios en Equipos de Emergencia</v>
+        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B137" t="str">
         <v/>
       </c>
       <c r="C137" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
+        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B138" t="str">
         <v/>
       </c>
       <c r="C138" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>PEMP, Plataformas, PRL</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
+        <v/>
       </c>
       <c r="B139" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C139" t="str">
-        <v>Manipulación Cargas, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B140" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C140" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B141" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C141" t="str">
-        <v>PEMP, Plataformas, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="142">
@@ -1971,7 +1971,7 @@
         <v/>
       </c>
       <c r="B142" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C142" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1982,7 +1982,7 @@
         <v/>
       </c>
       <c r="B143" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C143" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1993,7 +1993,7 @@
         <v/>
       </c>
       <c r="B144" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C144" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2004,7 +2004,7 @@
         <v/>
       </c>
       <c r="B145" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C145" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2015,7 +2015,7 @@
         <v/>
       </c>
       <c r="B146" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C146" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2026,7 +2026,7 @@
         <v/>
       </c>
       <c r="B147" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C147" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2037,7 +2037,7 @@
         <v/>
       </c>
       <c r="B148" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C148" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2048,7 +2048,7 @@
         <v/>
       </c>
       <c r="B149" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
       </c>
       <c r="C149" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2059,7 +2059,7 @@
         <v/>
       </c>
       <c r="B150" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C150" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2070,7 +2070,7 @@
         <v/>
       </c>
       <c r="B151" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C151" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2081,7 +2081,7 @@
         <v/>
       </c>
       <c r="B152" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C152" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="B153" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C153" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2103,7 +2103,7 @@
         <v/>
       </c>
       <c r="B154" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C154" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="B155" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C155" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2125,7 +2125,7 @@
         <v/>
       </c>
       <c r="B156" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C156" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2133,29 +2133,29 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v/>
+        <v>PRL SEGURIDAD VIAL</v>
       </c>
       <c r="B157" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="C157" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>PRL, Seguridad</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>PRL SEGURIDAD VIAL</v>
+        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
       </c>
       <c r="B158" t="str">
         <v/>
       </c>
       <c r="C158" t="str">
-        <v>PRL, Seguridad</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
+        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
       </c>
       <c r="B159" t="str">
         <v/>
@@ -2166,18 +2166,18 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
+        <v>PRODQUIM/000</v>
       </c>
       <c r="B160" t="str">
         <v/>
       </c>
       <c r="C160" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>PRODQUIM/000</v>
+        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B161" t="str">
         <v/>
@@ -2188,13 +2188,13 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v/>
       </c>
       <c r="B162" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C162" t="str">
-        <v>—</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="163">
@@ -2243,40 +2243,40 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
+        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B167" t="str">
         <v/>
       </c>
       <c r="C167" t="str">
-        <v>Espacios Confinados</v>
+        <v>—</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B168" t="str">
         <v/>
       </c>
       <c r="C168" t="str">
-        <v>—</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>RECICLAJE PARA FERRALLADO</v>
       </c>
       <c r="B169" t="str">
         <v/>
       </c>
       <c r="C169" t="str">
-        <v>Carretillas</v>
+        <v>—</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>RECICLAJE PARA FERRALLADO</v>
+        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B170" t="str">
         <v/>
@@ -2287,7 +2287,7 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B171" t="str">
         <v/>
@@ -2298,7 +2298,7 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B172" t="str">
         <v/>
@@ -2309,7 +2309,7 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B173" t="str">
         <v/>
@@ -2320,7 +2320,7 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B174" t="str">
         <v/>
@@ -2331,7 +2331,7 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B175" t="str">
         <v/>
@@ -2342,7 +2342,7 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B176" t="str">
         <v/>
@@ -2353,18 +2353,18 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>RECICLAJE PARA OPERADORES DE PUENTE-GRÚA</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B177" t="str">
         <v/>
       </c>
       <c r="C177" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>—</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B178" t="str">
         <v/>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
       </c>
       <c r="B179" t="str">
         <v/>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B180" t="str">
         <v/>
@@ -2397,24 +2397,24 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v/>
       </c>
       <c r="B181" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C181" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="B182" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C182" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="183">
@@ -2422,7 +2422,7 @@
         <v/>
       </c>
       <c r="B183" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C183" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2433,7 +2433,7 @@
         <v/>
       </c>
       <c r="B184" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C21- TRABAJOS DE INSTALACIONES, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES (TIC Y DIGITALIZACIÓN)</v>
       </c>
       <c r="C184" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2444,7 +2444,7 @@
         <v/>
       </c>
       <c r="B185" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C23- TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C185" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2455,7 +2455,7 @@
         <v/>
       </c>
       <c r="B186" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C21- TRABAJOS DE INSTALACIONES, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES (TIC Y DIGITALIZACIÓN)</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C186" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2466,7 +2466,7 @@
         <v/>
       </c>
       <c r="B187" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C23- TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C187" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2477,7 +2477,7 @@
         <v/>
       </c>
       <c r="B188" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C188" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2485,29 +2485,29 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v/>
+        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
       </c>
       <c r="B189" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v/>
       </c>
       <c r="C189" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v/>
+        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B190" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="C190" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
+        <v>REVESTIMIENTO DE YESO</v>
       </c>
       <c r="B191" t="str">
         <v/>
@@ -2518,46 +2518,46 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
       </c>
       <c r="B192" t="str">
         <v/>
       </c>
       <c r="C192" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>REVESTIMIENTO DE YESO</v>
+        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
       </c>
       <c r="B193" t="str">
         <v/>
       </c>
       <c r="C193" t="str">
-        <v>—</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
+        <v/>
       </c>
       <c r="B194" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C194" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
+        <v/>
       </c>
       <c r="B195" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C195" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="196">
@@ -2565,7 +2565,7 @@
         <v/>
       </c>
       <c r="B196" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C196" t="str">
         <v>Construcción, PRL</v>
@@ -2576,7 +2576,7 @@
         <v/>
       </c>
       <c r="B197" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C197" t="str">
         <v>Construcción, PRL</v>
@@ -2587,7 +2587,7 @@
         <v/>
       </c>
       <c r="B198" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="C198" t="str">
         <v>Construcción, PRL</v>
@@ -2598,7 +2598,7 @@
         <v/>
       </c>
       <c r="B199" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C199" t="str">
         <v>Construcción, PRL</v>
@@ -2609,7 +2609,7 @@
         <v/>
       </c>
       <c r="B200" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C200" t="str">
         <v>Construcción, PRL</v>
@@ -2620,7 +2620,7 @@
         <v/>
       </c>
       <c r="B201" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
       </c>
       <c r="C201" t="str">
         <v>Construcción, PRL</v>
@@ -2631,7 +2631,7 @@
         <v/>
       </c>
       <c r="B202" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C202" t="str">
         <v>Construcción, PRL</v>
@@ -2642,7 +2642,7 @@
         <v/>
       </c>
       <c r="B203" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C203" t="str">
         <v>Construcción, PRL</v>
@@ -2653,7 +2653,7 @@
         <v/>
       </c>
       <c r="B204" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C204" t="str">
         <v>Construcción, PRL</v>
@@ -2664,7 +2664,7 @@
         <v/>
       </c>
       <c r="B205" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C205" t="str">
         <v>Construcción, PRL</v>
@@ -2675,7 +2675,7 @@
         <v/>
       </c>
       <c r="B206" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C206" t="str">
         <v>Construcción, PRL</v>
@@ -2686,7 +2686,7 @@
         <v/>
       </c>
       <c r="B207" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C207" t="str">
         <v>Construcción, PRL</v>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="B208" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C208" t="str">
         <v>Construcción, PRL</v>
@@ -2708,7 +2708,7 @@
         <v/>
       </c>
       <c r="B209" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGON EN OBRA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C209" t="str">
         <v>Construcción, PRL</v>
@@ -2719,7 +2719,7 @@
         <v/>
       </c>
       <c r="B210" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C210" t="str">
         <v>Construcción, PRL</v>
@@ -2730,7 +2730,7 @@
         <v/>
       </c>
       <c r="B211" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="C211" t="str">
         <v>Construcción, PRL</v>
@@ -2741,7 +2741,7 @@
         <v/>
       </c>
       <c r="B212" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CIMENTACIONES ESPECIALES, SONDEOS Y PERFORACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C212" t="str">
         <v>Construcción, PRL</v>
@@ -2752,7 +2752,7 @@
         <v/>
       </c>
       <c r="B213" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C213" t="str">
         <v>Construcción, PRL</v>
@@ -2763,7 +2763,7 @@
         <v/>
       </c>
       <c r="B214" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
       </c>
       <c r="C214" t="str">
         <v>Construcción, PRL</v>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="B215" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C215" t="str">
         <v>Construcción, PRL</v>
@@ -2785,7 +2785,7 @@
         <v/>
       </c>
       <c r="B216" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C216" t="str">
         <v>Construcción, PRL</v>
@@ -2796,7 +2796,7 @@
         <v/>
       </c>
       <c r="B217" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C217" t="str">
         <v>Construcción, PRL</v>
@@ -2807,7 +2807,7 @@
         <v/>
       </c>
       <c r="B218" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C218" t="str">
         <v>Construcción, PRL</v>
@@ -2818,7 +2818,7 @@
         <v/>
       </c>
       <c r="B219" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C219" t="str">
         <v>Construcción, PRL</v>
@@ -2829,7 +2829,7 @@
         <v/>
       </c>
       <c r="B220" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGON EN OBRA</v>
       </c>
       <c r="C220" t="str">
         <v>Construcción, PRL</v>
@@ -2840,10 +2840,10 @@
         <v/>
       </c>
       <c r="B221" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C221" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="222">
@@ -2851,10 +2851,10 @@
         <v/>
       </c>
       <c r="B222" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C222" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="223">
@@ -2862,10 +2862,10 @@
         <v/>
       </c>
       <c r="B223" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C223" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="224">
@@ -2873,10 +2873,10 @@
         <v/>
       </c>
       <c r="B224" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGON EN OBRA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C224" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="225">
@@ -2884,7 +2884,7 @@
         <v/>
       </c>
       <c r="B225" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C225" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2895,10 +2895,10 @@
         <v/>
       </c>
       <c r="B226" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
       </c>
       <c r="C226" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Incendios, Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="227">
@@ -2906,7 +2906,7 @@
         <v/>
       </c>
       <c r="B227" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C227" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2917,7 +2917,7 @@
         <v/>
       </c>
       <c r="B228" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C228" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2928,7 +2928,7 @@
         <v/>
       </c>
       <c r="B229" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C229" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2939,7 +2939,7 @@
         <v/>
       </c>
       <c r="B230" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C230" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2950,7 +2950,7 @@
         <v/>
       </c>
       <c r="B231" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C231" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2961,7 +2961,7 @@
         <v/>
       </c>
       <c r="B232" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C232" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2972,10 +2972,10 @@
         <v/>
       </c>
       <c r="B233" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
       </c>
       <c r="C233" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Incendios, Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="234">
@@ -2983,7 +2983,7 @@
         <v/>
       </c>
       <c r="B234" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C234" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -2991,95 +2991,95 @@
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v/>
+        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
       </c>
       <c r="B235" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C235" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
       </c>
       <c r="B236" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C236" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
       </c>
       <c r="B237" t="str">
         <v/>
       </c>
       <c r="C237" t="str">
-        <v>Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
       </c>
       <c r="B238" t="str">
         <v/>
       </c>
       <c r="C238" t="str">
-        <v>Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
+        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
       </c>
       <c r="B239" t="str">
         <v/>
       </c>
       <c r="C239" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
+        <v>SEGURIDAD EN EL USO DE PLATAFORMAS ELEVADORAS. RECICLAJE</v>
       </c>
       <c r="B240" t="str">
         <v/>
       </c>
       <c r="C240" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>PEMP, Plataformas, Seguridad</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
+        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B241" t="str">
         <v/>
       </c>
       <c r="C241" t="str">
-        <v>Seguridad</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>SEGURIDAD EN EL USO DE PUENTES-GRÚA. RECICLAJE</v>
+        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
       </c>
       <c r="B242" t="str">
         <v/>
       </c>
       <c r="C242" t="str">
-        <v>Puente Grúa, Grúa, Seguridad</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B243" t="str">
         <v/>
@@ -3090,172 +3090,172 @@
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
       </c>
       <c r="B244" t="str">
         <v/>
       </c>
       <c r="C244" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
       </c>
       <c r="B245" t="str">
         <v/>
       </c>
       <c r="C245" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
       </c>
       <c r="B246" t="str">
         <v/>
       </c>
       <c r="C246" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
       </c>
       <c r="B247" t="str">
         <v/>
       </c>
       <c r="C247" t="str">
-        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
+        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
       </c>
       <c r="B248" t="str">
         <v/>
       </c>
       <c r="C248" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
+        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
       </c>
       <c r="B249" t="str">
         <v/>
       </c>
       <c r="C249" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Riesgo Químico, Seguridad</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
+        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
       </c>
       <c r="B250" t="str">
         <v/>
       </c>
       <c r="C250" t="str">
-        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
+        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
       </c>
       <c r="B251" t="str">
         <v/>
       </c>
       <c r="C251" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Grúa, Conducción Vehículos</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
+        <v>SOLADOS Y ALICATADOS</v>
       </c>
       <c r="B252" t="str">
         <v/>
       </c>
       <c r="C252" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B253" t="str">
         <v/>
       </c>
       <c r="C253" t="str">
-        <v>Riesgo Químico, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B254" t="str">
         <v/>
       </c>
       <c r="C254" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
+        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B255" t="str">
         <v/>
       </c>
       <c r="C255" t="str">
-        <v>Grúa, Conducción Vehículos</v>
+        <v>—</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>SOLADOS Y ALICATADOS</v>
+        <v/>
       </c>
       <c r="B256" t="str">
-        <v/>
+        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C256" t="str">
-        <v>—</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
       </c>
       <c r="B257" t="str">
         <v/>
       </c>
       <c r="C257" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v>TRABAJOS DE ARQUEOLOGÍA</v>
       </c>
       <c r="B258" t="str">
         <v/>
       </c>
       <c r="C258" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B259" t="str">
         <v/>
@@ -3266,18 +3266,18 @@
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v/>
+        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
       </c>
       <c r="B260" t="str">
-        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C260" t="str">
-        <v>Amianto</v>
+        <v>—</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
+        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
       </c>
       <c r="B261" t="str">
         <v/>
@@ -3288,29 +3288,29 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>TRABAJOS DE ARQUEOLOGÍA</v>
+        <v>TRABAJOS DE SOLDADURA</v>
       </c>
       <c r="B262" t="str">
         <v/>
       </c>
       <c r="C262" t="str">
-        <v>—</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
       </c>
       <c r="B263" t="str">
         <v/>
       </c>
       <c r="C263" t="str">
-        <v>—</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
       </c>
       <c r="B264" t="str">
         <v/>
@@ -3321,62 +3321,18 @@
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
       </c>
       <c r="B265" t="str">
         <v/>
       </c>
       <c r="C265" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="str">
-        <v>TRABAJOS DE SOLDADURA</v>
-      </c>
-      <c r="B266" t="str">
-        <v/>
-      </c>
-      <c r="C266" t="str">
-        <v>Soldadura</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="str">
-        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
-      </c>
-      <c r="B267" t="str">
-        <v/>
-      </c>
-      <c r="C267" t="str">
-        <v>Trabajos en Altura</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
-      </c>
-      <c r="B268" t="str">
-        <v/>
-      </c>
-      <c r="C268" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
-      </c>
-      <c r="B269" t="str">
-        <v/>
-      </c>
-      <c r="C269" t="str">
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C269"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C265"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: Actualización de datos Excel y diccionario de sinergias (15/06/2026)
</commit_message>
<xml_diff>
--- a/public/data/diccionario_sinergias_final.xlsx
+++ b/public/data/diccionario_sinergias_final.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C265"/>
+  <dimension ref="A1:C230"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -497,7 +497,7 @@
         <v>EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B8" t="str">
-        <v>EXTINCIÓN DE INCENDIOS CON INTERVENCIÓN Y EVACUACIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>EXTINCIÓN DE INCENDIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C8" t="str">
         <v>Extinción Incendios, Incendios</v>
@@ -505,43 +505,43 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EXTINCIÓN DE INCENDIOS Y PRIMEROS AUXILIOS</v>
+        <v>OPERADORES DE PLATAFORMAS ELEVADORAS</v>
       </c>
       <c r="B9" t="str">
-        <v>EXTINCIÓN DE INCENDIOS. TEÓRICO-PRÁCTICO</v>
+        <v>MANEJO SEGURO DE PLATAFORMAS ELEVADORAS SEGÚN NORMA UNE 58923:2020. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C9" t="str">
-        <v>Extinción Incendios, Incendios</v>
+        <v>PEMP, Plataformas</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v>EXTINCIÓN DE INCENDIOS Y PRIMEROS AUXILIOS</v>
       </c>
       <c r="B10" t="str">
-        <v>MANEJO SEGURO DE PLATAFORMAS ELEVADORAS SEGÚN NORMA UNE 58923:2020. TEÓRICO-PRÁCTICO</v>
+        <v>PREVENCIÓN Y EXTINCIÓN DE INCENDIOS PARA EQUIPOS DE PRIMERA INTERVENCIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C10" t="str">
-        <v>PEMP, Plataformas</v>
+        <v>Extinción Incendios, Incendios</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
+        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
       </c>
       <c r="B11" t="str">
-        <v>PREVENCIÓN Y EXTINCIÓN DE INCENDIOS PARA EQUIPOS DE PRIMERA INTERVENCIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="C11" t="str">
-        <v>Extinción Incendios, Incendios</v>
+        <v>Puente Grúa, Grúa</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>MANEJO SEGURO DE PUENTE GRÚA</v>
+        <v>OPERADORES DE PUENTE-GRÚA</v>
       </c>
       <c r="B12" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C28 - OPERADORES DE PUENTE-GRÚA</v>
+        <v>SEGURIDAD EN EL MANEJO PUENTES-GRÚA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C12" t="str">
         <v>Puente Grúa, Grúa</v>
@@ -549,43 +549,43 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>OPERADOR DE PUENTE GRÚA Y POLIPASTOS</v>
+        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B13" t="str">
-        <v>SEGURIDAD EN EL MANEJO PUENTES-GRÚA. TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C13" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de premontaje, montaje, cambio de formato y ensamblaje en fábricas</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
       </c>
       <c r="B14" t="str">
-        <v>NIVEL BÁSICO PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA</v>
+        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C14" t="str">
-        <v>Metal, PRL, Nivel Básico</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>PRL PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B15" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C15" t="str">
-        <v>Carretillas, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B16" t="str">
-        <v>RECICLAJE EN SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C16" t="str">
         <v>Carretillas, Seguridad</v>
@@ -593,274 +593,274 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SEGURIDAD EN TRABAJOS CON PLATAFORMA SUSPENDIDA PARA TRABAJOS EN GRÚA PORTAINER Y ADIESTRAMIENTO EQUIPO DE EVACUACIÓN ALTURAS</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B17" t="str">
-        <v>SEGURIDAD EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C17" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLA ELEVADORA, TRANSPALETA Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
       </c>
       <c r="B18" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS FRONTALES TEÓRICO-PRÁCTICO</v>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C18" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B19" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE CARRETILLAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
+        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C19" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
       </c>
       <c r="B20" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="C20" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SEGURIDAD EN TRABAJOS EL ALTURA</v>
+        <v>ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B21" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C21" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ALTURAS TELCO I</v>
+        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
       </c>
       <c r="B22" t="str">
-        <v>ALTURAS TELCO I. TEÓRICO-PRÁCTICO</v>
+        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C22" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
+        <v>PRIMEROS AUXILIOS</v>
       </c>
       <c r="B23" t="str">
-        <v>ALTURAS TELCO II. TEÓRICO-PRÁCTICO</v>
+        <v>FORMACION AELEC EN PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C23" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>ALTURAS TELCO I</v>
       </c>
       <c r="B24" t="str">
-        <v>CARRETILLAS ELEVADORAS (CARNET DE CARRETILLERO). TEÓRICO-PRÁCTICO</v>
+        <v>FORMACIÓN TRABAJOS EN ALTURA NIVEL 1. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C24" t="str">
-        <v>Carretillas</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
+        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
       </c>
       <c r="B25" t="str">
-        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
+        <v>NIVEL BASICO DE PREVENCION DE LAS ACTIVIDADES DEL METAL EN LA CONSTRUCCION</v>
       </c>
       <c r="C25" t="str">
-        <v>Carretillas</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA SOBRE MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
       </c>
       <c r="B26" t="str">
-        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
       </c>
       <c r="C26" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Metal, Nivel Básico</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ESPACIOS CONFINADOS TELCO</v>
+        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
       </c>
       <c r="B27" t="str">
-        <v>ESPACIOS CONFINADOS TELCO. TEÓRICO-PRÁCTICO</v>
+        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C27" t="str">
-        <v>Espacios Confinados</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
+        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
       </c>
       <c r="B28" t="str">
-        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
+        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C28" t="str">
-        <v>Espacios Confinados</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
+        <v>Primeros Auxilios en Equipos de Emergencia</v>
       </c>
       <c r="B29" t="str">
-        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C29" t="str">
-        <v>Espacios Confinados</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>PRIMEROS AUXILIOS</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
       </c>
       <c r="B30" t="str">
-        <v>FORMACION AELEC EN PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C30" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
       </c>
       <c r="B31" t="str">
-        <v>NIVEL BASICO DE PREVENCION DE LAS ACTIVIDADES DEL METAL EN LA CONSTRUCCION</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C31" t="str">
-        <v>Construcción, Nivel Básico</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
+        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B32" t="str">
-        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C32" t="str">
-        <v>Metal, Nivel Básico</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
+        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
       </c>
       <c r="B33" t="str">
-        <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="C33" t="str">
-        <v>Carretillas</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>PRIMEROS AUXILIOS PEDIÁTRICO</v>
+        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
       </c>
       <c r="B34" t="str">
-        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="C34" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
+        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B35" t="str">
-        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C35" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
       </c>
       <c r="B36" t="str">
-        <v>PRL EN ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C36" t="str">
-        <v>Espacios Confinados</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>RECICLAJE  ALTURAS TELCO I</v>
+        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="B37" t="str">
-        <v>PRL EN TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
       </c>
       <c r="C37" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Formación en PRL para operarios de almacén según Art. 32 del Convenio Colectivo del Comercio del Metal de la Provincia de Alicante</v>
+        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
       </c>
       <c r="B38" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>RECICLAJE RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C38" t="str">
-        <v>Metal, PRL</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
+        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
       </c>
       <c r="B39" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>RIESGO ELÉCTRICO . TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C39" t="str">
-        <v>Metal, PRL</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
+        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B40" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>RIESGO ELÉCTRICO RD 614/2001. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C40" t="str">
-        <v>Metal, PRL</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES ELÉCTRICAS DE ALTA Y BAJA TENSIÓN</v>
+        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
       </c>
       <c r="B41" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C15 - INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C41" t="str">
         <v>Riesgo Eléctrico</v>
@@ -868,274 +868,274 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
+        <v>RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B42" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C42" t="str">
-        <v>Carretillas</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
       </c>
       <c r="B43" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C43" t="str">
-        <v>Soldadura</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
+        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
       </c>
       <c r="B44" t="str">
-        <v>RECICLAJE DE CURSO DE TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C44" t="str">
-        <v>Amianto</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
       </c>
       <c r="B45" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C45" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
       </c>
       <c r="B46" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C4 - OPERARIOS EN TRABAJOS DE SOLDADURA Y OXICORTE</v>
+        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C46" t="str">
-        <v>Soldadura</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
+        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B47" t="str">
-        <v>RIESGO ELÉCTRICO . TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C47" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
+        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B48" t="str">
-        <v>RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C48" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>RECICLAJE PARA INSTALADORES Y REPARADORES DE LÍNEAS Y EQUIPOS ELÉCTRICOS</v>
+        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="B49" t="str">
-        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C49" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B50" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C50" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
+        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B51" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C51" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>RIESGO ELÉCTRICO TELCO</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B52" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C52" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B53" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="C53" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
+        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B54" t="str">
-        <v>SEGURIDAD CONTRA INCENDIOS Y ACTUACIÓN ANTE EMERGENCIAS. TEÓRICO-PRÁCTICO.</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C54" t="str">
-        <v>Incendios, Seguridad</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA</v>
+        <v>ACOSO LABORAL Y SEXUAL</v>
       </c>
       <c r="B55" t="str">
-        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C55" t="str">
-        <v>Trabajos en Altura</v>
+        <v>—</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>ADMINISTRATIVOS</v>
       </c>
       <c r="B56" t="str">
-        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
+        <v/>
       </c>
       <c r="C56" t="str">
-        <v>Construcción</v>
+        <v>—</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>ALBAÑILERÍA</v>
       </c>
       <c r="B57" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v/>
       </c>
       <c r="C57" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
+        <v>CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B58" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="C58" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>CONDUCCIÓN SEGURA</v>
       </c>
       <c r="B59" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v/>
       </c>
       <c r="C59" t="str">
-        <v>Metal</v>
+        <v>Conducción</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>CONDUCTORES Y TRANSPORTISTAS</v>
       </c>
       <c r="B60" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v/>
       </c>
       <c r="C60" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="B61" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v/>
       </c>
       <c r="C61" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>OTROS OFICIOS DEL METAL</v>
+        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
       </c>
       <c r="B62" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
+        <v/>
       </c>
       <c r="C62" t="str">
-        <v>Metal</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="B63" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v/>
       </c>
       <c r="C63" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>ENCOFRADOS</v>
       </c>
       <c r="B64" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v/>
       </c>
       <c r="C64" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
+        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
       </c>
       <c r="B65" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="C65" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>ACOSO LABORAL Y SEXUAL</v>
+        <v/>
       </c>
       <c r="B66" t="str">
-        <v/>
+        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
       </c>
       <c r="C66" t="str">
         <v>—</v>
@@ -1143,18 +1143,18 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>ADMINISTRATIVOS</v>
+        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
       </c>
       <c r="B67" t="str">
         <v/>
       </c>
       <c r="C67" t="str">
-        <v>—</v>
+        <v>Extinción Incendios, Incendios, Nivel Básico</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>ALBAÑILERÍA</v>
+        <v>FERRALLADO</v>
       </c>
       <c r="B68" t="str">
         <v/>
@@ -1165,7 +1165,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Campaña Allive 80.0 Fase II-Técnico de Prevención por un día-EL ALTO</v>
+        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B69" t="str">
         <v/>
@@ -1176,43 +1176,43 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>CARPINTERÍA METÁLICA</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
       </c>
       <c r="B70" t="str">
         <v/>
       </c>
       <c r="C70" t="str">
-        <v>—</v>
+        <v>PRL, Nivel Básico</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>CONDUCCIÓN SEGURA</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
       </c>
       <c r="B71" t="str">
         <v/>
       </c>
       <c r="C71" t="str">
-        <v>Conducción</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>CONDUCTORES Y TRANSPORTISTAS</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
       </c>
       <c r="B72" t="str">
         <v/>
       </c>
       <c r="C72" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v/>
       </c>
       <c r="B73" t="str">
-        <v/>
+        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C73" t="str">
         <v>—</v>
@@ -1220,7 +1220,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
       </c>
       <c r="B74" t="str">
         <v/>
@@ -1231,18 +1231,18 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
+        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
       </c>
       <c r="B75" t="str">
         <v/>
       </c>
       <c r="C75" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B76" t="str">
         <v/>
@@ -1253,7 +1253,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>ENCOFRADOS</v>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
       </c>
       <c r="B77" t="str">
         <v/>
@@ -1264,7 +1264,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
+        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
       </c>
       <c r="B78" t="str">
         <v/>
@@ -1275,7 +1275,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>ESTABILIZACIÓN DE EXPLANADAS Y EXTENDIDO DE FIRMES</v>
+        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B79" t="str">
         <v/>
@@ -1286,10 +1286,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v/>
+        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
       </c>
       <c r="B80" t="str">
-        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
+        <v/>
       </c>
       <c r="C80" t="str">
         <v>—</v>
@@ -1297,7 +1297,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>FERRALLADO</v>
+        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B81" t="str">
         <v/>
@@ -1308,7 +1308,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v>MANIPULACION DE ALIMENTOS</v>
       </c>
       <c r="B82" t="str">
         <v/>
@@ -1319,10 +1319,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>FORMACIÓN DE RIESGOS ESPECÍFICOS EN EL SECTOR DE PRODUCCIÓN</v>
+        <v/>
       </c>
       <c r="B83" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS</v>
       </c>
       <c r="C83" t="str">
         <v>—</v>
@@ -1330,54 +1330,54 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>FORMACIÓN EN SEGURIDAD EN LAS GRÚAS AUTOMÁTICAS DEL TREN</v>
+        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B84" t="str">
         <v/>
       </c>
       <c r="C84" t="str">
-        <v>Grúa, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
+        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B85" t="str">
         <v/>
       </c>
       <c r="C85" t="str">
-        <v>PRL, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
+        <v>MEDIDAS DE EMERGENCIA</v>
       </c>
       <c r="B86" t="str">
         <v/>
       </c>
       <c r="C86" t="str">
-        <v>PRL</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
+        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="B87" t="str">
         <v/>
       </c>
       <c r="C87" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v/>
+        <v>MONTAJE ANDAMIOS APOYADOS</v>
       </c>
       <c r="B88" t="str">
-        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C88" t="str">
         <v>—</v>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
+        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
       </c>
       <c r="B89" t="str">
         <v/>
@@ -1396,10 +1396,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
+        <v/>
       </c>
       <c r="B90" t="str">
-        <v/>
+        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C90" t="str">
         <v>—</v>
@@ -1410,15 +1410,15 @@
         <v/>
       </c>
       <c r="B91" t="str">
-        <v>INFECCIONES RESPIRATORIAS AGUDAS</v>
+        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
       </c>
       <c r="C91" t="str">
-        <v>—</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v>OPERACIONES TELCO</v>
       </c>
       <c r="B92" t="str">
         <v/>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
+        <v>OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B93" t="str">
         <v/>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
+        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B94" t="str">
         <v/>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B95" t="str">
         <v/>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
+        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
       </c>
       <c r="B96" t="str">
         <v/>
@@ -1473,7 +1473,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B97" t="str">
         <v/>
@@ -1484,7 +1484,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>MANIPULACION DE ALIMENTOS</v>
+        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B98" t="str">
         <v/>
@@ -1495,10 +1495,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v/>
+        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B99" t="str">
-        <v>MANIPULADOR DE ALIMENTOS</v>
+        <v/>
       </c>
       <c r="C99" t="str">
         <v>—</v>
@@ -1506,10 +1506,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v/>
+        <v>OTRO TIPO DE INSTALACIONES</v>
       </c>
       <c r="B100" t="str">
-        <v>MANIPULADOR DE ALIMENTOS. RESTAURACIÓN</v>
+        <v/>
       </c>
       <c r="C100" t="str">
         <v>—</v>
@@ -1517,7 +1517,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>PINTURA</v>
       </c>
       <c r="B101" t="str">
         <v/>
@@ -1528,18 +1528,18 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>MANTENIMIENTO, REPARACIÓN E INSTALACIÓN DE ASCENSORES</v>
+        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
       </c>
       <c r="B102" t="str">
         <v/>
       </c>
       <c r="C102" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
       </c>
       <c r="B103" t="str">
         <v/>
@@ -1550,65 +1550,65 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>MEDIDAS DE EMERGENCIA</v>
+        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
       </c>
       <c r="B104" t="str">
         <v/>
       </c>
       <c r="C104" t="str">
-        <v>Emergencias</v>
+        <v>Ergonomía, PRL</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
       </c>
       <c r="B105" t="str">
         <v/>
       </c>
       <c r="C105" t="str">
-        <v>—</v>
+        <v>Grúa, PRL</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>MONTAJE ANDAMIOS APOYADOS</v>
+        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B106" t="str">
         <v/>
       </c>
       <c r="C106" t="str">
-        <v>—</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
+        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
       </c>
       <c r="B107" t="str">
         <v/>
       </c>
       <c r="C107" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v/>
+        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
       </c>
       <c r="B108" t="str">
-        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C108" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>OPERACIONES TELCO</v>
+        <v/>
       </c>
       <c r="B109" t="str">
-        <v/>
+        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C109" t="str">
         <v>—</v>
@@ -1616,79 +1616,79 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>OPERADOR DE CAMIÓN GRÚA</v>
+        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B110" t="str">
         <v/>
       </c>
       <c r="C110" t="str">
-        <v>Grúa</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>OPERADOR DE PALA CARGADORA</v>
+        <v/>
       </c>
       <c r="B111" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C111" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="B112" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C112" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>OPERADORES DE PUENTE-GRÚA</v>
+        <v/>
       </c>
       <c r="B113" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C113" t="str">
-        <v>Puente Grúa, Grúa</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v/>
       </c>
       <c r="B114" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C114" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v/>
       </c>
       <c r="B115" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C115" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>OPERARIO DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGÓN, DE MACHAQUEO Y CLASIFICACIÓN DE ÁRIDOS</v>
+        <v/>
       </c>
       <c r="B116" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C116" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="117">
@@ -1696,395 +1696,395 @@
         <v/>
       </c>
       <c r="B117" t="str">
-        <v>OPERARIO DE LA CONSTRUCCION EN VIRTUD DEL CONTENIDO DE LA LEY 31/95 DE 8 DE NOVIEMBRE (ART. 19)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
       </c>
       <c r="C117" t="str">
-        <v>Construcción</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
+        <v/>
       </c>
       <c r="B118" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C118" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="B119" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C119" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="B120" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C120" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="B121" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C121" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v/>
       </c>
       <c r="B122" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C122" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>OTRO TIPO DE INSTALACIONES</v>
+        <v/>
       </c>
       <c r="B123" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="C123" t="str">
-        <v>—</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>PINTURA</v>
+        <v/>
       </c>
       <c r="B124" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C124" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
+        <v/>
       </c>
       <c r="B125" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
       </c>
       <c r="C125" t="str">
-        <v>Emergencias</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>PRÁCTICAS EN LAS NORMAS DE SEGURIDAD EN EL USO DE PEMP</v>
+        <v/>
       </c>
       <c r="B126" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C126" t="str">
-        <v>PEMP, Seguridad</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
+        <v/>
       </c>
       <c r="B127" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C127" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
+        <v/>
       </c>
       <c r="B128" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C128" t="str">
-        <v>Ergonomía, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
+        <v/>
       </c>
       <c r="B129" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C129" t="str">
-        <v>Grúa, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B130" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C130" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA CONTRATAS DEL GRUPO ENCE</v>
+        <v/>
       </c>
       <c r="B131" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C131" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
+        <v>PRODQUIM/000</v>
       </c>
       <c r="B132" t="str">
         <v/>
       </c>
       <c r="C132" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
+        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B133" t="str">
         <v/>
       </c>
       <c r="C133" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v/>
+        <v>RECICLAJE  ALTURAS TELCO I</v>
       </c>
       <c r="B134" t="str">
-        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C134" t="str">
-        <v>—</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Primeros Auxilios en Equipos de Emergencia</v>
+        <v/>
       </c>
       <c r="B135" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C135" t="str">
-        <v>Primeros Auxilios, Emergencias</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>PRL EN MANIPULACION MANUAL DE CARGAS - TRANSPALETA</v>
+        <v/>
       </c>
       <c r="B136" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C136" t="str">
-        <v>Manipulación Cargas, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B137" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C137" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>PRL PARA OPERADORES DE PLATAFORMAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B138" t="str">
-        <v/>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C138" t="str">
-        <v>PEMP, Plataformas, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v/>
+        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B139" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C139" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v/>
+        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B140" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v/>
       </c>
       <c r="C140" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v/>
+        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B141" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v/>
       </c>
       <c r="C141" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v/>
+        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B142" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="C142" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v/>
+        <v>RECICLAJE PARA FERRALLADO</v>
       </c>
       <c r="B143" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v/>
       </c>
       <c r="C143" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v/>
+        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B144" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C144" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v/>
+        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B145" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v/>
       </c>
       <c r="C145" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v/>
+        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B146" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="C146" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v/>
+        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B147" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v/>
       </c>
       <c r="C147" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v/>
+        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B148" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v/>
       </c>
       <c r="C148" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v/>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B149" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
+        <v/>
       </c>
       <c r="C149" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v/>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B150" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C25 - TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v/>
       </c>
       <c r="C150" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v/>
+        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B151" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v/>
       </c>
       <c r="C151" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v/>
+        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B152" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="C152" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="153">
@@ -2092,7 +2092,7 @@
         <v/>
       </c>
       <c r="B153" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C153" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2103,7 +2103,7 @@
         <v/>
       </c>
       <c r="B154" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C154" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="B155" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C155" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2125,7 +2125,7 @@
         <v/>
       </c>
       <c r="B156" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C21- TRABAJOS DE INSTALACIONES, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES (TIC Y DIGITALIZACIÓN)</v>
       </c>
       <c r="C156" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -2133,57 +2133,57 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>PRL SEGURIDAD VIAL</v>
+        <v/>
       </c>
       <c r="B157" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C23- TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C157" t="str">
-        <v>PRL, Seguridad</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MANEJO DE MÁQUINA TELESCÓPICA</v>
+        <v/>
       </c>
       <c r="B158" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C25- TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C158" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>PRL TEÓRICO-PRÁCTICO EN MOTOSIERRA Y DESBROZADORA</v>
+        <v/>
       </c>
       <c r="B159" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C159" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>PRODQUIM/000</v>
+        <v/>
       </c>
       <c r="B160" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C160" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v/>
       </c>
       <c r="B161" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C161" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="162">
@@ -2191,32 +2191,32 @@
         <v/>
       </c>
       <c r="B162" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>RECICLAJE PRL TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C14- TRABAJOS DE INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C162" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v/>
+        <v>REVESTIMIENTO DE YESO</v>
       </c>
       <c r="B163" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C163" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v/>
+        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
       </c>
       <c r="B164" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C164" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="165">
@@ -2224,175 +2224,175 @@
         <v/>
       </c>
       <c r="B165" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C165" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v/>
       </c>
       <c r="B166" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C166" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="B167" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C167" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B168" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C168" t="str">
-        <v>Carretillas</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>RECICLAJE PARA FERRALLADO</v>
+        <v/>
       </c>
       <c r="B169" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C169" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="B170" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C170" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v/>
       </c>
       <c r="B171" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
       </c>
       <c r="C171" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="B172" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C172" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v/>
       </c>
       <c r="B173" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C173" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v/>
       </c>
       <c r="B174" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C174" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>RECICLAJE PARA OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="B175" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C175" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="B176" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C176" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="B177" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C177" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="B178" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C178" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN TRABAJOS DE JOYERÍA</v>
+        <v/>
       </c>
       <c r="B179" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C179" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="B180" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C180" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="181">
@@ -2400,10 +2400,10 @@
         <v/>
       </c>
       <c r="B181" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C181" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="182">
@@ -2411,10 +2411,10 @@
         <v/>
       </c>
       <c r="B182" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C182" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="183">
@@ -2422,10 +2422,10 @@
         <v/>
       </c>
       <c r="B183" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
       </c>
       <c r="C183" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="184">
@@ -2433,10 +2433,10 @@
         <v/>
       </c>
       <c r="B184" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C21- TRABAJOS DE INSTALACIONES, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES (TIC Y DIGITALIZACIÓN)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C184" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="185">
@@ -2444,10 +2444,10 @@
         <v/>
       </c>
       <c r="B185" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C23- TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C185" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="186">
@@ -2455,10 +2455,10 @@
         <v/>
       </c>
       <c r="B186" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C186" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="187">
@@ -2466,10 +2466,10 @@
         <v/>
       </c>
       <c r="B187" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C187" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="188">
@@ -2477,65 +2477,65 @@
         <v/>
       </c>
       <c r="B188" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C188" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>RECICLAJE RECICLAJE PARA RESPONSABLES DE OBRA Y TÉCNICOS DE EJECUCIÓN</v>
+        <v/>
       </c>
       <c r="B189" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
       </c>
       <c r="C189" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>RECICLAJE SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
+        <v/>
       </c>
       <c r="B190" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
       </c>
       <c r="C190" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>REVESTIMIENTO DE YESO</v>
+        <v/>
       </c>
       <c r="B191" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C191" t="str">
-        <v>—</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
+        <v/>
       </c>
       <c r="B192" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C192" t="str">
-        <v>—</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
+        <v/>
       </c>
       <c r="B193" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C193" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="194">
@@ -2543,10 +2543,10 @@
         <v/>
       </c>
       <c r="B194" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C194" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="195">
@@ -2554,10 +2554,10 @@
         <v/>
       </c>
       <c r="B195" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C195" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="196">
@@ -2565,10 +2565,10 @@
         <v/>
       </c>
       <c r="B196" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C196" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="197">
@@ -2576,10 +2576,10 @@
         <v/>
       </c>
       <c r="B197" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C197" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="198">
@@ -2587,10 +2587,10 @@
         <v/>
       </c>
       <c r="B198" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C198" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="199">
@@ -2598,10 +2598,10 @@
         <v/>
       </c>
       <c r="B199" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C199" t="str">
-        <v>Construcción, PRL</v>
+        <v>Riesgo Eléctrico, Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="200">
@@ -2609,10 +2609,10 @@
         <v/>
       </c>
       <c r="B200" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C200" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="201">
@@ -2620,10 +2620,10 @@
         <v/>
       </c>
       <c r="B201" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C201" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="202">
@@ -2631,10 +2631,10 @@
         <v/>
       </c>
       <c r="B202" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C202" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="203">
@@ -2642,131 +2642,131 @@
         <v/>
       </c>
       <c r="B203" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C203" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v/>
+        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
       </c>
       <c r="B204" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v/>
       </c>
       <c r="C204" t="str">
-        <v>Construcción, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
       </c>
       <c r="B205" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v/>
       </c>
       <c r="C205" t="str">
-        <v>Construcción, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
       </c>
       <c r="B206" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v/>
       </c>
       <c r="C206" t="str">
-        <v>Construcción, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
       </c>
       <c r="B207" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
+        <v/>
       </c>
       <c r="C207" t="str">
-        <v>Construcción, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B208" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C208" t="str">
-        <v>Construcción, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v/>
+        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B209" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v/>
       </c>
       <c r="C209" t="str">
-        <v>Construcción, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v/>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
       </c>
       <c r="B210" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
+        <v/>
       </c>
       <c r="C210" t="str">
-        <v>Construcción, PRL</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v/>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
       </c>
       <c r="B211" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v/>
       </c>
       <c r="C211" t="str">
-        <v>Construcción, PRL</v>
+        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v/>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
       </c>
       <c r="B212" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v/>
       </c>
       <c r="C212" t="str">
-        <v>Construcción, PRL</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v/>
+        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B213" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v/>
       </c>
       <c r="C213" t="str">
-        <v>Construcción, PRL</v>
+        <v>Extinción Incendios, Incendios, Seguridad</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v/>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
       </c>
       <c r="B214" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
+        <v/>
       </c>
       <c r="C214" t="str">
-        <v>Construcción, PRL</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="215">
@@ -2774,10 +2774,10 @@
         <v/>
       </c>
       <c r="B215" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGURIDAD EN TRABAJOS EN ESAPCIOS CONFINADOS. NIVEL 1. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C215" t="str">
-        <v>Construcción, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="216">
@@ -2785,554 +2785,169 @@
         <v/>
       </c>
       <c r="B216" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGURIDAD Y MANEJO CON PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C216" t="str">
-        <v>Construcción, PRL</v>
+        <v>PEMP, Plataformas, Seguridad</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v/>
+        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
       </c>
       <c r="B217" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v/>
       </c>
       <c r="C217" t="str">
-        <v>Construcción, PRL</v>
+        <v>Riesgo Químico, Seguridad</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v/>
+        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
       </c>
       <c r="B218" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v/>
       </c>
       <c r="C218" t="str">
-        <v>Construcción, PRL</v>
+        <v>Grúa, Conducción Vehículos</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v/>
+        <v>SOLADOS Y ALICATADOS</v>
       </c>
       <c r="B219" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v/>
       </c>
       <c r="C219" t="str">
-        <v>Construcción, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v/>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B220" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGON EN OBRA</v>
+        <v/>
       </c>
       <c r="C220" t="str">
-        <v>Construcción, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v/>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B221" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C221" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v/>
+        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B222" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C222" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v/>
+        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
       </c>
       <c r="B223" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v/>
       </c>
       <c r="C223" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v/>
+        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B224" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C224" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v/>
+        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
       </c>
       <c r="B225" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C225" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v/>
+        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
       </c>
       <c r="B226" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
+        <v/>
       </c>
       <c r="C226" t="str">
-        <v>Incendios, Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v/>
+        <v>TRABAJOS DE SOLDADURA</v>
       </c>
       <c r="B227" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C227" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v/>
+        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
       </c>
       <c r="B228" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C228" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v/>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
       </c>
       <c r="B229" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C229" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v/>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
       </c>
       <c r="B230" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v/>
       </c>
       <c r="C230" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="str">
-        <v/>
-      </c>
-      <c r="B231" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
-      </c>
-      <c r="C231" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="str">
-        <v/>
-      </c>
-      <c r="B232" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
-      </c>
-      <c r="C232" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="str">
-        <v/>
-      </c>
-      <c r="B233" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE EQUIPOS CONTRAINCENDIOS</v>
-      </c>
-      <c r="C233" t="str">
-        <v>Incendios, Sector Metal, Construcción, Metal, PRL</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="str">
-        <v/>
-      </c>
-      <c r="B234" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
-      </c>
-      <c r="C234" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="str">
-        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
-      </c>
-      <c r="B235" t="str">
-        <v/>
-      </c>
-      <c r="C235" t="str">
-        <v>Seguridad</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="str">
-        <v>SEGURIDAD EN EL MANEJO DE PALA CARGADORA</v>
-      </c>
-      <c r="B236" t="str">
-        <v/>
-      </c>
-      <c r="C236" t="str">
-        <v>Seguridad</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
-      </c>
-      <c r="B237" t="str">
-        <v/>
-      </c>
-      <c r="C237" t="str">
-        <v>Carretillas, Seguridad</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
-      </c>
-      <c r="B238" t="str">
-        <v/>
-      </c>
-      <c r="C238" t="str">
-        <v>Carretillas, Seguridad</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="str">
-        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
-      </c>
-      <c r="B239" t="str">
-        <v/>
-      </c>
-      <c r="C239" t="str">
-        <v>Seguridad</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="str">
-        <v>SEGURIDAD EN EL USO DE PLATAFORMAS ELEVADORAS. RECICLAJE</v>
-      </c>
-      <c r="B240" t="str">
-        <v/>
-      </c>
-      <c r="C240" t="str">
-        <v>PEMP, Plataformas, Seguridad</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="str">
-        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
-      </c>
-      <c r="B241" t="str">
-        <v/>
-      </c>
-      <c r="C241" t="str">
-        <v>Carretillas, Seguridad</v>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="str">
-        <v>SEGURIDAD EN EL USO Y MANEJO DE TRANSPALETAS MANUALES, ELÉCTRICAS Y APLILADORES</v>
-      </c>
-      <c r="B242" t="str">
-        <v/>
-      </c>
-      <c r="C242" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="str">
-        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
-      </c>
-      <c r="B243" t="str">
-        <v/>
-      </c>
-      <c r="C243" t="str">
-        <v>Carretillas, Seguridad</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
-      </c>
-      <c r="B244" t="str">
-        <v/>
-      </c>
-      <c r="C244" t="str">
-        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
-      </c>
-      <c r="B245" t="str">
-        <v/>
-      </c>
-      <c r="C245" t="str">
-        <v>Espacios Confinados, Seguridad</v>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL BÁSICO</v>
-      </c>
-      <c r="B246" t="str">
-        <v/>
-      </c>
-      <c r="C246" t="str">
-        <v>Trabajos en Altura, Nivel Básico, Seguridad</v>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
-      </c>
-      <c r="B247" t="str">
-        <v/>
-      </c>
-      <c r="C247" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="str">
-        <v>SEGURIDAD PARA CONTRATAS Y TRABAJADORES DE ILBOC</v>
-      </c>
-      <c r="B248" t="str">
-        <v/>
-      </c>
-      <c r="C248" t="str">
-        <v>Seguridad</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
-      </c>
-      <c r="B249" t="str">
-        <v/>
-      </c>
-      <c r="C249" t="str">
-        <v>Riesgo Químico, Seguridad</v>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="str">
-        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
-      </c>
-      <c r="B250" t="str">
-        <v/>
-      </c>
-      <c r="C250" t="str">
-        <v>Riesgo Eléctrico, Seguridad</v>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="str">
-        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
-      </c>
-      <c r="B251" t="str">
-        <v/>
-      </c>
-      <c r="C251" t="str">
-        <v>Grúa, Conducción Vehículos</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="str">
-        <v>SOLADOS Y ALICATADOS</v>
-      </c>
-      <c r="B252" t="str">
-        <v/>
-      </c>
-      <c r="C252" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
-      </c>
-      <c r="B253" t="str">
-        <v/>
-      </c>
-      <c r="C253" t="str">
-        <v>DEA, Nivel Básico</v>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
-      </c>
-      <c r="B254" t="str">
-        <v/>
-      </c>
-      <c r="C254" t="str">
-        <v>DEA, Nivel Básico</v>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="str">
-        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
-      </c>
-      <c r="B255" t="str">
-        <v/>
-      </c>
-      <c r="C255" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="str">
-        <v/>
-      </c>
-      <c r="B256" t="str">
-        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
-      </c>
-      <c r="C256" t="str">
-        <v>Amianto</v>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="str">
-        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
-      </c>
-      <c r="B257" t="str">
-        <v/>
-      </c>
-      <c r="C257" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="str">
-        <v>TRABAJOS DE ARQUEOLOGÍA</v>
-      </c>
-      <c r="B258" t="str">
-        <v/>
-      </c>
-      <c r="C258" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="str">
-        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
-      </c>
-      <c r="B259" t="str">
-        <v/>
-      </c>
-      <c r="C259" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="str">
-        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
-      </c>
-      <c r="B260" t="str">
-        <v/>
-      </c>
-      <c r="C260" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="str">
-        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
-      </c>
-      <c r="B261" t="str">
-        <v/>
-      </c>
-      <c r="C261" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="str">
-        <v>TRABAJOS DE SOLDADURA</v>
-      </c>
-      <c r="B262" t="str">
-        <v/>
-      </c>
-      <c r="C262" t="str">
-        <v>Soldadura</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="str">
-        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
-      </c>
-      <c r="B263" t="str">
-        <v/>
-      </c>
-      <c r="C263" t="str">
-        <v>Trabajos en Altura</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
-      </c>
-      <c r="B264" t="str">
-        <v/>
-      </c>
-      <c r="C264" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
-      </c>
-      <c r="B265" t="str">
-        <v/>
-      </c>
-      <c r="C265" t="str">
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C265"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C230"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update app with new training data and synergy dictionary (June 22, 2026)
</commit_message>
<xml_diff>
--- a/public/data/diccionario_sinergias_final.xlsx
+++ b/public/data/diccionario_sinergias_final.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C230"/>
+  <dimension ref="A1:C214"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -626,32 +626,32 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
+        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
       </c>
       <c r="B20" t="str">
-        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
+        <v>CONDUCCIÓN Y MANEJO SEGURO DE CARRETILLAS ELEVADORAS SEGÚN NORMA UNE 58451:2016</v>
       </c>
       <c r="C20" t="str">
-        <v>Manipulación Cargas</v>
+        <v>Carretillas</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ESPACIOS CONFINADOS TELCO</v>
+        <v>RIESGOS Y MEDIDAS PREVENTIVAS EN LA MANIPULACIÓN Y MOVIMIENTO DE CARGAS</v>
       </c>
       <c r="B21" t="str">
-        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
+        <v>CUIDADO DE LA ESPALDA EN LA MANIPULACIÓN MANUAL DE CARGAS</v>
       </c>
       <c r="C21" t="str">
-        <v>Espacios Confinados</v>
+        <v>Manipulación Cargas</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
+        <v>ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B22" t="str">
-        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
+        <v>ESPACIOS CONFINADOS Y ATMÓSFERAS EXPLOSIVAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C22" t="str">
         <v>Espacios Confinados</v>
@@ -659,51 +659,51 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>PRIMEROS AUXILIOS</v>
+        <v>JORNADAS FORMATIVAS DE TRABAJO EN ESPACIOS CONFINADOS PARA Z.O. LOTE 3</v>
       </c>
       <c r="B23" t="str">
-        <v>FORMACION AELEC EN PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>ESPACIOS CONFINADOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C23" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ALTURAS TELCO I</v>
+        <v>PRIMEROS AUXILIOS</v>
       </c>
       <c r="B24" t="str">
-        <v>FORMACIÓN TRABAJOS EN ALTURA NIVEL 1. TEÓRICO-PRÁCTICO</v>
+        <v>FORMACION AELEC EN PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C24" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Primeros Auxilios</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
+        <v>ALTURAS TELCO I</v>
       </c>
       <c r="B25" t="str">
-        <v>NIVEL BASICO DE PREVENCION DE LAS ACTIVIDADES DEL METAL EN LA CONSTRUCCION</v>
+        <v>FORMACIÓN TRABAJOS EN ALTURA NIVEL 1. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C25" t="str">
-        <v>Construcción, Nivel Básico</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
+        <v>NIVEL BÁSICO DE PREVENCIÓN EN LA CONSTRUCCIÓN 60 H</v>
       </c>
       <c r="B26" t="str">
-        <v>NIVEL BÁSICO DEL SECTOR METAL DE LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (50 H): DELEGADOS DE PREVENCIÓN</v>
+        <v>NIVEL BASICO DE PREVENCION DE LAS ACTIVIDADES DEL METAL EN LA CONSTRUCCION</v>
       </c>
       <c r="C26" t="str">
-        <v>Metal, Nivel Básico</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>FORMACIÓN INICIAL OPERADOR DE CARRETILLAS DE MANUTENCIÓN HASTA 10.000 kg SEGÚN UNE 58451:2016, Categoría II Tipo 4: Carret. elev. mástil carga voladizo</v>
+        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B27" t="str">
         <v>OPERADORES DE CARRETILLAS DE MANUTENCIÓN DE HASTA 10.000 KG. TEÓRICO-PRÁCTICO</v>
@@ -717,7 +717,7 @@
         <v>PRIMEROS AUXILIOS Y EMERGENCIAS</v>
       </c>
       <c r="B28" t="str">
-        <v>PRIMEROS AUXILIOS EN LA EMPRESA. TEÓRICO-PRÁCTICO</v>
+        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C28" t="str">
         <v>Primeros Auxilios</v>
@@ -725,13 +725,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Primeros Auxilios en Equipos de Emergencia</v>
+        <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en actividades de tratamientos superficiales de las piezas del metal: desengrasado, limpieza, decapado, recubrimiento, pintura.</v>
       </c>
       <c r="B29" t="str">
-        <v>PRIMEROS AUXILIOS. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C29" t="str">
-        <v>Primeros Auxilios</v>
+        <v>Metal, PRL</v>
       </c>
     </row>
     <row r="30">
@@ -739,7 +739,7 @@
         <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Operarios en almacén y logística y aprovisionamiento en los procesos de fabricación</v>
       </c>
       <c r="B30" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C14 - TRABAJOS INSTALACIÓN, MANTENIMIENTO-REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C30" t="str">
         <v>Metal, PRL</v>
@@ -750,7 +750,7 @@
         <v>Nivel Básico en Prevención de Riesgos Laborales en el Metal. Oficio: Talleres de reparación de vehículos</v>
       </c>
       <c r="B31" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C31" t="str">
         <v>Metal, PRL</v>
@@ -758,7 +758,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>FORMACIÓN PRÁCTICA DE 2 HORAS EN EL MANEJO DE CARRETILLAS ELEVADORAS</v>
+        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
       </c>
       <c r="B32" t="str">
         <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
@@ -780,7 +780,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>FORMACIÓN PRÁCTICA Y TEÓRICA DE APILADOR, CARRETILLA Y TRANSPALETA</v>
+        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B34" t="str">
         <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C27 - CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
@@ -827,7 +827,7 @@
         <v>MANEJO SEGURO DE TRANSPALETAS ELEVADORAS ELÉCTRICAS</v>
       </c>
       <c r="B38" t="str">
-        <v>RECICLAJE RIESGO ELÉCTRICO TELCO. TEÓRICO-PRÁCTICO</v>
+        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C38" t="str">
         <v>Riesgo Eléctrico</v>
@@ -838,7 +838,7 @@
         <v>RECICLAJE PARA ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE A.T. Y B.T.</v>
       </c>
       <c r="B39" t="str">
-        <v>RIESGO ELÉCTRICO . TEÓRICO-PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C39" t="str">
         <v>Riesgo Eléctrico</v>
@@ -849,7 +849,7 @@
         <v>RECICLAJE RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B40" t="str">
-        <v>RIESGO ELÉCTRICO RD 614/2001. TEÓRICO-PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C40" t="str">
         <v>Riesgo Eléctrico</v>
@@ -860,7 +860,7 @@
         <v>RIESGO ELÉCTRICO EN BAJA TENSIÓN: CAPACITACIÓN PARA TRABAJADORES AUTORIZADOS SEGÚN R.D. 614/2001</v>
       </c>
       <c r="B41" t="str">
-        <v>RIESGOS ELÉCTRICOS EN ALTA Y BAJA TENSIÓN. TEÓRICO-PRÁCTICO</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C41" t="str">
         <v>Riesgo Eléctrico</v>
@@ -871,7 +871,7 @@
         <v>RIESGO ELÉCTRICO TELCO</v>
       </c>
       <c r="B42" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
       </c>
       <c r="C42" t="str">
         <v>Riesgo Eléctrico</v>
@@ -879,54 +879,54 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
+        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
       </c>
       <c r="B43" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C43" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
+        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B44" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C44" t="str">
-        <v>Riesgo Eléctrico</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>FORMACIÓN INICIAL PREVENTIVA PARA OPERARIOS DE TRABAJOS CON AMIANTO EN ESCENARIOS DE RIESGO MAYOR UNE 171370-1</v>
+        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="B45" t="str">
-        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C45" t="str">
-        <v>Amianto</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>FORMACIÓN TEÓRICO PRÁCTICA DE TRABAJOS EN ALTURA</v>
+        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="B46" t="str">
-        <v>TRABAJOS EN ALTURA. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C46" t="str">
-        <v>Trabajos en Altura</v>
+        <v>Metal</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>METAL: INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B47" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C47" t="str">
         <v>Metal</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>METAL: INSTALACIÓN DE ASCENSORES</v>
+        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B48" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C48" t="str">
         <v>Metal</v>
@@ -945,10 +945,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>METAL: TRABAJOS EN INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="B49" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C49" t="str">
         <v>Metal</v>
@@ -956,10 +956,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
       </c>
       <c r="B50" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C14 -TRABAJOS INSTALACIÓN, MANTENIMIENTO- REPARACIÓN EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C50" t="str">
         <v>Metal</v>
@@ -967,10 +967,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
       </c>
       <c r="B51" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C51" t="str">
         <v>Metal</v>
@@ -978,40 +978,40 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>ACOSO LABORAL Y SEXUAL</v>
       </c>
       <c r="B52" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v/>
       </c>
       <c r="C52" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DEL METAL: DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA.</v>
+        <v>ADMINISTRATIVOS</v>
       </c>
       <c r="B53" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v/>
       </c>
       <c r="C53" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>RECICLAJE PARA OTROS OFICIOS DEL METAL</v>
+        <v>ALBAÑILERÍA</v>
       </c>
       <c r="B54" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v/>
       </c>
       <c r="C54" t="str">
-        <v>Metal</v>
+        <v>—</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ACOSO LABORAL Y SEXUAL</v>
+        <v>CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B55" t="str">
         <v/>
@@ -1022,18 +1022,18 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ADMINISTRATIVOS</v>
+        <v>CONDUCCIÓN SEGURA</v>
       </c>
       <c r="B56" t="str">
         <v/>
       </c>
       <c r="C56" t="str">
-        <v>—</v>
+        <v>Conducción</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ALBAÑILERÍA</v>
+        <v>CONDUCTORES Y TRANSPORTISTAS</v>
       </c>
       <c r="B57" t="str">
         <v/>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>CARPINTERÍA METÁLICA</v>
+        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="B58" t="str">
         <v/>
@@ -1055,18 +1055,18 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>CONDUCCIÓN SEGURA</v>
+        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
       </c>
       <c r="B59" t="str">
         <v/>
       </c>
       <c r="C59" t="str">
-        <v>Conducción</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>CONDUCTORES Y TRANSPORTISTAS</v>
+        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="B60" t="str">
         <v/>
@@ -1077,7 +1077,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>ENCOFRADOS</v>
       </c>
       <c r="B61" t="str">
         <v/>
@@ -1088,21 +1088,21 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>CURSO PARA DELEGADOS/AS Y MIEMBROS DE COMITÉS DE SEGURIDAD Y SALUD DE ANDALUCÍA</v>
+        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
       </c>
       <c r="B62" t="str">
         <v/>
       </c>
       <c r="C62" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v/>
       </c>
       <c r="B63" t="str">
-        <v/>
+        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
       </c>
       <c r="C63" t="str">
         <v>—</v>
@@ -1110,18 +1110,18 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>ENCOFRADOS</v>
+        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
       </c>
       <c r="B64" t="str">
         <v/>
       </c>
       <c r="C64" t="str">
-        <v>—</v>
+        <v>Extinción Incendios, Incendios, Nivel Básico</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>EQUIPOS DE PROTECCIÓN INDIVIDUAL. SELECCIÓN, USO Y CONSERVACIÓN</v>
+        <v>FERRALLADO</v>
       </c>
       <c r="B65" t="str">
         <v/>
@@ -1132,10 +1132,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v/>
+        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B66" t="str">
-        <v>ESTRES TÉRMICO EN EL ÁMBITO LABORAL</v>
+        <v/>
       </c>
       <c r="C66" t="str">
         <v>—</v>
@@ -1143,32 +1143,32 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>EXTINCIÓN DE INCENDIOS: NIVEL BÁSICO-EQUIPO PRIMERA INTERVENCIÓN</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
       </c>
       <c r="B67" t="str">
         <v/>
       </c>
       <c r="C67" t="str">
-        <v>Extinción Incendios, Incendios, Nivel Básico</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>FERRALLADO</v>
+        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
       </c>
       <c r="B68" t="str">
         <v/>
       </c>
       <c r="C68" t="str">
-        <v>—</v>
+        <v>PRL</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="B69" t="str">
-        <v/>
+        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C69" t="str">
         <v>—</v>
@@ -1176,43 +1176,43 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (BÁSICO CONTRATISTAS REPSOL</v>
+        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
       </c>
       <c r="B70" t="str">
         <v/>
       </c>
       <c r="C70" t="str">
-        <v>PRL, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE ERAS/ERSA</v>
+        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
       </c>
       <c r="B71" t="str">
         <v/>
       </c>
       <c r="C71" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>FORMACION PRL PARA CONTRATAS DE REPSOL (USO DE EXTINTORES</v>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B72" t="str">
         <v/>
       </c>
       <c r="C72" t="str">
-        <v>PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v/>
+        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
       </c>
       <c r="B73" t="str">
-        <v>HIGIENE POSTURAL .TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C73" t="str">
         <v>—</v>
@@ -1220,7 +1220,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>IGUALDAD DE GÉNERO Y SENSIBILIZACIÓN EN IGUALDAD Y NO DISCRIMINACIÓN AL COLECTIVO LGTBI</v>
+        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
       </c>
       <c r="B74" t="str">
         <v/>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>IMPLANTACIÓN DEL PLAN DE AUTOPROTECCIÓN</v>
+        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B75" t="str">
         <v/>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
       </c>
       <c r="B76" t="str">
         <v/>
@@ -1253,7 +1253,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES</v>
+        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
       </c>
       <c r="B77" t="str">
         <v/>
@@ -1264,7 +1264,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>MADERA Y MUEBLE: INSTALADOR DE ELEMENTOS DE CARPINTERÍA Y MUEBLE</v>
+        <v>MANIPULACION DE ALIMENTOS</v>
       </c>
       <c r="B78" t="str">
         <v/>
@@ -1275,10 +1275,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>MADERA Y MUEBLE: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v/>
       </c>
       <c r="B79" t="str">
-        <v/>
+        <v>MANIPULADOR DE ALIMENTOS</v>
       </c>
       <c r="C79" t="str">
         <v>—</v>
@@ -1286,7 +1286,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>MADERA: INSTALADOR DE ELEMENTOS DE CARPINTERÍA DE MADERA Y MUEBLE</v>
+        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B80" t="str">
         <v/>
@@ -1297,7 +1297,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>MADERA: MONTADOR DE ESTRUCTURAS DE MADERA</v>
+        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B81" t="str">
         <v/>
@@ -1308,21 +1308,21 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>MANIPULACION DE ALIMENTOS</v>
+        <v>MEDIDAS DE EMERGENCIA</v>
       </c>
       <c r="B82" t="str">
         <v/>
       </c>
       <c r="C82" t="str">
-        <v>—</v>
+        <v>Emergencias</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v/>
+        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
       </c>
       <c r="B83" t="str">
-        <v>MANIPULADOR DE ALIMENTOS</v>
+        <v/>
       </c>
       <c r="C83" t="str">
         <v>—</v>
@@ -1330,7 +1330,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>MANTENIMIENTO - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE LA INDUSTRIA SIDERÚRGICA  Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
       </c>
       <c r="B84" t="str">
         <v/>
@@ -1341,10 +1341,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v/>
       </c>
       <c r="B85" t="str">
-        <v/>
+        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C85" t="str">
         <v>—</v>
@@ -1352,18 +1352,18 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>MEDIDAS DE EMERGENCIA</v>
+        <v/>
       </c>
       <c r="B86" t="str">
-        <v/>
+        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
       </c>
       <c r="C86" t="str">
-        <v>Emergencias</v>
+        <v>Construcción, Nivel Básico</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>MONTADOR DE ESCAYOLA, PLACAS DE YESO LAMINADO Y ASIMILADOS</v>
+        <v>OPERACIONES TELCO</v>
       </c>
       <c r="B87" t="str">
         <v/>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>MONTAJE ANDAMIOS APOYADOS</v>
+        <v>OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="B88" t="str">
         <v/>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>MOVILIZACIÓN DE ENFERMOS. HIGIENE POSTURAL PARA LA PREVENCIÓN DE LAS ALTERACIONES MUSCULOESQUELÉTICAS</v>
+        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B89" t="str">
         <v/>
@@ -1396,10 +1396,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v/>
+        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="B90" t="str">
-        <v>MOVILIZACIÓN EN EL DOMICILIO. TEÓRICO-PRÁCTICO</v>
+        <v/>
       </c>
       <c r="C90" t="str">
         <v>—</v>
@@ -1407,18 +1407,18 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v/>
+        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
       </c>
       <c r="B91" t="str">
-        <v>NIVEL BASICO DE PREVENCION EN CONSTRUCCION</v>
+        <v/>
       </c>
       <c r="C91" t="str">
-        <v>Construcción, Nivel Básico</v>
+        <v>—</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>OPERACIONES TELCO</v>
+        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B92" t="str">
         <v/>
@@ -1429,7 +1429,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>OPERADORES DE APARATOS ELEVADORES</v>
+        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B93" t="str">
         <v/>
@@ -1440,7 +1440,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>OPERADORES DE VEHICULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B94" t="str">
         <v/>
@@ -1451,7 +1451,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>OTRO TIPO DE INSTALACIONES</v>
       </c>
       <c r="B95" t="str">
         <v/>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>OPERARIO DE TALLER DE MATERIALES: PIEDRAS INDUSTRIALES, TRATAMIENTO O TRANSFORMACIÓN DE MATERIALES, CANTEROS Y SIMILARES</v>
+        <v>PINTURA</v>
       </c>
       <c r="B96" t="str">
         <v/>
@@ -1473,7 +1473,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
       </c>
       <c r="B97" t="str">
         <v/>
@@ -1484,32 +1484,32 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
       </c>
       <c r="B98" t="str">
         <v/>
       </c>
       <c r="C98" t="str">
-        <v>—</v>
+        <v>Ergonomía, PRL</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B99" t="str">
         <v/>
       </c>
       <c r="C99" t="str">
-        <v>—</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>OTRO TIPO DE INSTALACIONES</v>
+        <v/>
       </c>
       <c r="B100" t="str">
-        <v/>
+        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C100" t="str">
         <v>—</v>
@@ -1517,90 +1517,90 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>PINTURA</v>
+        <v>Primeros Auxilios en Equipos de Emergencia</v>
       </c>
       <c r="B101" t="str">
         <v/>
       </c>
       <c r="C101" t="str">
-        <v>—</v>
+        <v>Primeros Auxilios, Emergencias</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>PLAN DE EMERGENCIA DEL COMPLEJO INDUSTRIAL DE REPSOL PETROLEO CARTAGENA</v>
+        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
       </c>
       <c r="B102" t="str">
         <v/>
       </c>
       <c r="C102" t="str">
-        <v>Emergencias</v>
+        <v>ATEX, PRL</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>PREPARACIÓN, REALIZACIÓN Y EVALUACIÓN DE SIMULACROS</v>
+        <v/>
       </c>
       <c r="B103" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C103" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>PREVENCION DE RIESGOS ERGONÓMICOS ASOCIADOS A TRABAJOS DE LIMPIEZA Y PUESTA A PUNTO DE HABITACIONES EN ESTABLECIMIENTOS HOTELEROS</v>
+        <v/>
       </c>
       <c r="B104" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C104" t="str">
-        <v>Ergonomía, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES ASOCIADOS AL USO DE GRÚA STS EN LABORES DE MANTENIMIENTO</v>
+        <v/>
       </c>
       <c r="B105" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C105" t="str">
-        <v>Grúa, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>PREVENCION DE RIESGOS LABORALES EN TRABAJOS CON PRESENCIA DE ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B106" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C106" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>PREVENCIÓN DE RIESGOS LABORALES PARA PERSONAL DE TALLER DE MANTENIMIENTO</v>
+        <v/>
       </c>
       <c r="B107" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C107" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>PREVENCIÓN FRENTE AL RIESGO POR EXPOSICIÓN A SÍLICE CRISTALINA RESPIRABLE EN INDUSTRIAS EXTRACTIVAS</v>
+        <v/>
       </c>
       <c r="B108" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C108" t="str">
-        <v>PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="109">
@@ -1608,21 +1608,21 @@
         <v/>
       </c>
       <c r="B109" t="str">
-        <v>PREVENCION LESIONES OSTEOMUSCULARES Y MEJORA DE LA SALUD. TEÓRICO-PRÁCTICO</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
       </c>
       <c r="C109" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>PRL EN TRABAJOS PRESENCIA ATMOSFERAS EXPLOSIVAS</v>
+        <v/>
       </c>
       <c r="B110" t="str">
-        <v/>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C110" t="str">
-        <v>ATEX, PRL</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="111">
@@ -1630,10 +1630,10 @@
         <v/>
       </c>
       <c r="B111" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
       </c>
       <c r="C111" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="112">
@@ -1641,7 +1641,7 @@
         <v/>
       </c>
       <c r="B112" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
       </c>
       <c r="C112" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1652,7 +1652,7 @@
         <v/>
       </c>
       <c r="B113" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C5-6- OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
       </c>
       <c r="C113" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1663,7 +1663,7 @@
         <v/>
       </c>
       <c r="B114" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="C114" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1674,7 +1674,7 @@
         <v/>
       </c>
       <c r="B115" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C115" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1685,7 +1685,7 @@
         <v/>
       </c>
       <c r="B116" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (20 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C116" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1696,7 +1696,7 @@
         <v/>
       </c>
       <c r="B117" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C1.1-A) - CNAE 24, OPERARIOS EN TRABAJOS DE PRODUCCIÓN EN LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
       </c>
       <c r="C117" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1707,7 +1707,7 @@
         <v/>
       </c>
       <c r="B118" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C118" t="str">
         <v>Sector Metal, Metal, PRL</v>
@@ -1715,35 +1715,35 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v/>
+        <v>PRODQUIM/000</v>
       </c>
       <c r="B119" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C12 - TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v/>
       </c>
       <c r="C119" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v/>
+        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
       </c>
       <c r="B120" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C13 - TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="C120" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v/>
+        <v>RECICLAJE  ALTURAS TELCO I</v>
       </c>
       <c r="B121" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C16 - TRABAJOS DE FONTANERÍA, INSTALACIONES DE CALEFACCIÓN-CLIMATIZACIÓN, INSTALACIONES DE AGUA CALIENTE SANITARIA E INSTALACIONES SOLARES TÉRMICAS</v>
+        <v/>
       </c>
       <c r="C121" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="122">
@@ -1751,10 +1751,10 @@
         <v/>
       </c>
       <c r="B122" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C19 - TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C122" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="123">
@@ -1762,7 +1762,7 @@
         <v/>
       </c>
       <c r="B123" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C2 - CNAE 30.1 Y 33.15, TRABAJOS DE CONSTRUCCIÓN, REPARACIÓN Y MANTENIMIENTO NAVAL EN ASTILLEROS Y MUELLES</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C123" t="str">
         <v>Sector Metal, Construcción, Metal, PRL</v>
@@ -1773,10 +1773,10 @@
         <v/>
       </c>
       <c r="B124" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C23 - TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C124" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="125">
@@ -1784,81 +1784,81 @@
         <v/>
       </c>
       <c r="B125" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C24 - TRABAJOS DE RECUPERACIÓN Y RECICLAJE DE MATERIAS PRIMAS SECUNDARIAS METÁLICAS</v>
+        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C125" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v/>
+        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B126" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C26 - CONDUCTORES/TRANSPORTISTAS</v>
+        <v/>
       </c>
       <c r="C126" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v/>
+        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
       </c>
       <c r="B127" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C30 - OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="C127" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Espacios Confinados</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v/>
+        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B128" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v/>
       </c>
       <c r="C128" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v/>
+        <v>RECICLAJE PARA FERRALLADO</v>
       </c>
       <c r="B129" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v/>
       </c>
       <c r="C129" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v/>
+        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="B130" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C8 - OPERARIOS EN ACTIVIDADES DE TRATAMIENTOS SUPERFICIALES DE LAS PIEZAS DE METAL  (DESENGRASADO, LIMPIEZA, DECAPADO, RECUBRIMIENTO, PINTURA)</v>
+        <v/>
       </c>
       <c r="C130" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v/>
+        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
       </c>
       <c r="B131" t="str">
-        <v>PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO (8 HORAS): C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="C131" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>PRODQUIM/000</v>
+        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="B132" t="str">
         <v/>
@@ -1869,7 +1869,7 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>PRODUCCIÓN - ACTIVIDADES DEL CNAE 24 RELATIVAS A LAS PERSONAS TRABAJADORAS DE  LA INDUSTRIA SIDERÚRGICA Y DE PRIMERA TRANSFORMACIÓN DEL ACERO</v>
+        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
       </c>
       <c r="B133" t="str">
         <v/>
@@ -1880,150 +1880,150 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>RECICLAJE  ALTURAS TELCO I</v>
+        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B134" t="str">
         <v/>
       </c>
       <c r="C134" t="str">
-        <v>Trabajos en Altura</v>
+        <v>—</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v/>
+        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="B135" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C135" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v/>
+        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="B136" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C136" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v/>
+        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
       </c>
       <c r="B137" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C137" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v/>
+        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B138" t="str">
-        <v>RECICLAJE DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN: TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C138" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>RECICLAJE EN SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
+        <v/>
       </c>
       <c r="B139" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C139" t="str">
-        <v>DEA, Nivel Básico</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>RECICLAJE ESPACIOS CONFINADOS TELCO</v>
+        <v/>
       </c>
       <c r="B140" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
       </c>
       <c r="C140" t="str">
-        <v>Espacios Confinados</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>RECICLAJE PARA CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="B141" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="C141" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>RECICLAJE PARA CONDUCTORES DE CARRETILLAS ELEVADORAS</v>
+        <v/>
       </c>
       <c r="B142" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C25- TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
       </c>
       <c r="C142" t="str">
-        <v>Carretillas</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>RECICLAJE PARA FERRALLADO</v>
+        <v/>
       </c>
       <c r="B143" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
       </c>
       <c r="C143" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>RECICLAJE PARA FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="B144" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
       </c>
       <c r="C144" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>RECICLAJE PARA INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DEPÓSITOS AUXILIARES; EQUIPOS DE TECNOLOGÍAS DE TELECOMUNICACIONES Y DE LA INFORMACIÓN, REDES DE INFORMACIÓN Y DATOS</v>
+        <v/>
       </c>
       <c r="B145" t="str">
-        <v/>
+        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
       </c>
       <c r="C145" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>RECICLAJE PARA INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="B146" t="str">
-        <v/>
+        <v>RECICLAJE PRL TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C14- TRABAJOS DE INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
       </c>
       <c r="C146" t="str">
-        <v>—</v>
+        <v>Sector Metal, Metal, PRL</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>RECICLAJE PARA MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC).</v>
+        <v>REVESTIMIENTO DE YESO</v>
       </c>
       <c r="B147" t="str">
         <v/>
@@ -2034,18 +2034,18 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>RECICLAJE PARA MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>RIESGO ELÉCTRICO: PROTOCOLO DE ACTUACIÓN DE IBERDROLA: REEX Y ETC-09 RIESGO ELÉCTRICO</v>
       </c>
       <c r="B148" t="str">
         <v/>
       </c>
       <c r="C148" t="str">
-        <v>—</v>
+        <v>Riesgo Eléctrico</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>RECICLAJE PARA OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
       </c>
       <c r="B149" t="str">
         <v/>
@@ -2056,35 +2056,35 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v/>
       </c>
       <c r="B150" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C150" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>RECICLAJE PARA OPERARIOS EN ALMACÉN Y LOGÍSTICA Y APROVISIONAMIENTO EN LOS PROCESOS DE FABRICACIÓN</v>
+        <v/>
       </c>
       <c r="B151" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C151" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>RECICLAJE PARA TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v/>
       </c>
       <c r="B152" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C152" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="153">
@@ -2092,10 +2092,10 @@
         <v/>
       </c>
       <c r="B153" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C10 - TRABAJOS DE CARPINTERÍA METÁLICA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C153" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="154">
@@ -2103,10 +2103,10 @@
         <v/>
       </c>
       <c r="B154" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C12-TRABAJOS DE MECÁNICA, MANTENIMIENTO Y REPARACIÓN DE MÁQUINAS, EQUIPOS INDUSTRIALES Y/O EQUIPOS ELECTROMECÁNICOS (INDUSTRIA AEROESPACIAL, ETC.)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C154" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="155">
@@ -2114,10 +2114,10 @@
         <v/>
       </c>
       <c r="B155" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C13- TRABAJOS EN TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C155" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="156">
@@ -2125,10 +2125,10 @@
         <v/>
       </c>
       <c r="B156" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C21- TRABAJOS DE INSTALACIONES, MANTENIMIENTO Y REPARACIÓN DE INFRAESTRUCTURAS DE TELECOMUNICACIONES (TIC Y DIGITALIZACIÓN)</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
       </c>
       <c r="C156" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="157">
@@ -2136,10 +2136,10 @@
         <v/>
       </c>
       <c r="B157" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C23- TRABAJOS DE OTRO TIPO DE INSTALACIONES TALES COMO INSTALACIONES SOLARES FOTOVOLTAICAS O INSTALACIONES EÓLICAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C157" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="158">
@@ -2147,10 +2147,10 @@
         <v/>
       </c>
       <c r="B158" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C25- TRABAJOS DE CONTROL DE CALIDAD, VERIFICACIÓN E INSPECCIÓN DE MATERIAS EN CURSO DE FABRICACIÓN Y EN PRODUCTOS TERMINADOS DEL SECTOR</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C158" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="159">
@@ -2158,10 +2158,10 @@
         <v/>
       </c>
       <c r="B159" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C5-6 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR ARRANQUE DE VIRUTA O POR ABRASIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C159" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="160">
@@ -2169,10 +2169,10 @@
         <v/>
       </c>
       <c r="B160" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C7 - OPERARIOS DE MÁQUINAS DE MECANIZADO POR DEFORMACIÓN Y CORTE DEL METAL</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C160" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="161">
@@ -2180,10 +2180,10 @@
         <v/>
       </c>
       <c r="B161" t="str">
-        <v>RECICLAJE PRL PARA TRABAJADORES SECTOR METAL EN LAS AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C9 - OPERARIOS EN ACTIVIDADES DE PREMONTAJE, MONTAJE, CAMBIO DE FORMATO Y ENSAMBLAJE EN FÁBRICAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C161" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="162">
@@ -2191,32 +2191,32 @@
         <v/>
       </c>
       <c r="B162" t="str">
-        <v>RECICLAJE PRL TRABAJADORES SECTOR METAL EN AREAS DE PRODUCCIÓN Y/O MANTENIMIENTO: C14- TRABAJOS DE INSTALACIÓN, MANTENIMIENTO Y REPARACIÓN DE EQUIPOS INFORMÁTICOS, AUTOMATISMOS Y SU PROGRAMACIÓN, ORDENADORES Y SUS PERIFÉRICOS O DISPOSITIVOS AUXILIARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
       </c>
       <c r="C162" t="str">
-        <v>Sector Metal, Metal, PRL</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>REVESTIMIENTO DE YESO</v>
+        <v/>
       </c>
       <c r="B163" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
       </c>
       <c r="C163" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>RIESGOS HIGIÉNICOS EN EL CENTRO DE TRABAJO. RESULTADOS MEDICIONES HIGIÉNICAS</v>
+        <v/>
       </c>
       <c r="B164" t="str">
-        <v/>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
       </c>
       <c r="C164" t="str">
-        <v>—</v>
+        <v>Construcción, PRL</v>
       </c>
     </row>
     <row r="165">
@@ -2224,7 +2224,7 @@
         <v/>
       </c>
       <c r="B165" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
       </c>
       <c r="C165" t="str">
         <v>Construcción, PRL</v>
@@ -2235,7 +2235,7 @@
         <v/>
       </c>
       <c r="B166" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="C166" t="str">
         <v>Construcción, PRL</v>
@@ -2246,7 +2246,7 @@
         <v/>
       </c>
       <c r="B167" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
       </c>
       <c r="C167" t="str">
         <v>Construcción, PRL</v>
@@ -2257,7 +2257,7 @@
         <v/>
       </c>
       <c r="B168" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERARIOS DE INSTALACIONES TEMPORALES DE OBRA Y AUXILIARES: PLANTAS DE AGLOMERADO, DE HORMIGON, DE MACHAQUEO Y CLASIFICACION DE ARIDOS</v>
       </c>
       <c r="C168" t="str">
         <v>Construcción, PRL</v>
@@ -2268,7 +2268,7 @@
         <v/>
       </c>
       <c r="B169" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
       </c>
       <c r="C169" t="str">
         <v>Construcción, PRL</v>
@@ -2279,7 +2279,7 @@
         <v/>
       </c>
       <c r="B170" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
       </c>
       <c r="C170" t="str">
         <v>Construcción, PRL</v>
@@ -2290,7 +2290,7 @@
         <v/>
       </c>
       <c r="B171" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
       </c>
       <c r="C171" t="str">
         <v>Construcción, PRL</v>
@@ -2301,7 +2301,7 @@
         <v/>
       </c>
       <c r="B172" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
       </c>
       <c r="C172" t="str">
         <v>Construcción, PRL</v>
@@ -2312,7 +2312,7 @@
         <v/>
       </c>
       <c r="B173" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
       </c>
       <c r="C173" t="str">
         <v>Construcción, PRL</v>
@@ -2323,7 +2323,7 @@
         <v/>
       </c>
       <c r="B174" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
       </c>
       <c r="C174" t="str">
         <v>Construcción, PRL</v>
@@ -2334,7 +2334,7 @@
         <v/>
       </c>
       <c r="B175" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
       </c>
       <c r="C175" t="str">
         <v>Construcción, PRL</v>
@@ -2345,7 +2345,7 @@
         <v/>
       </c>
       <c r="B176" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
       </c>
       <c r="C176" t="str">
         <v>Construcción, PRL</v>
@@ -2356,10 +2356,10 @@
         <v/>
       </c>
       <c r="B177" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ALBAÑILERÍA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C177" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="178">
@@ -2367,10 +2367,10 @@
         <v/>
       </c>
       <c r="B178" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): APARATOS ELEVADORES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C178" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="179">
@@ -2378,10 +2378,10 @@
         <v/>
       </c>
       <c r="B179" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): CONSERVACIÓN Y EXPLOTACIÓN DE CARRETERAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C179" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="180">
@@ -2389,10 +2389,10 @@
         <v/>
       </c>
       <c r="B180" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): ENCOFRADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C180" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="181">
@@ -2400,10 +2400,10 @@
         <v/>
       </c>
       <c r="B181" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): MONTAJE DE ESTRUCTURAS TUBULARES</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C181" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="182">
@@ -2411,10 +2411,10 @@
         <v/>
       </c>
       <c r="B182" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): OPERADORES DE VEHÍCULOS Y MAQUINARIA DE MOVIMIENTO DE TIERRAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C182" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="183">
@@ -2422,10 +2422,10 @@
         <v/>
       </c>
       <c r="B183" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): PINTURA</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
       </c>
       <c r="C183" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="184">
@@ -2433,10 +2433,10 @@
         <v/>
       </c>
       <c r="B184" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): SOLADOS Y ALICATADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
       </c>
       <c r="C184" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="185">
@@ -2444,10 +2444,10 @@
         <v/>
       </c>
       <c r="B185" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE CONSTRUCCION Y MANTENIMIENTO DE VIAS FERREAS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
       </c>
       <c r="C185" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="186">
@@ -2455,10 +2455,10 @@
         <v/>
       </c>
       <c r="B186" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE DEMOLICIÓN Y REHABILITACIÓN</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
       </c>
       <c r="C186" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="187">
@@ -2466,10 +2466,10 @@
         <v/>
       </c>
       <c r="B187" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FABRICACIÓN Y MONTAJE DE ELEMENTOS PREFABRICADOS</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
       </c>
       <c r="C187" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="188">
@@ -2477,109 +2477,109 @@
         <v/>
       </c>
       <c r="B188" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERIA E INSTALACIONES DE CLIMATIZACION</v>
+        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
       </c>
       <c r="C188" t="str">
-        <v>Construcción, PRL</v>
+        <v>Sector Metal, Construcción, Metal, PRL</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v/>
+        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
       </c>
       <c r="B189" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
+        <v/>
       </c>
       <c r="C189" t="str">
-        <v>Construcción, PRL</v>
+        <v>Seguridad</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
       </c>
       <c r="B190" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DE LA MADERA EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALADOR DE ELEMENTOS DE CARPINTERIA Y MUEBLE</v>
+        <v/>
       </c>
       <c r="C190" t="str">
-        <v>Construcción, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
       </c>
       <c r="B191" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C191" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v/>
+        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
       </c>
       <c r="B192" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v/>
       </c>
       <c r="C192" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v/>
+        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
       </c>
       <c r="B193" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v/>
       </c>
       <c r="C193" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Carretillas, Seguridad</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v/>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
       </c>
       <c r="B194" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C194" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v/>
+        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
       </c>
       <c r="B195" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C195" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Espacios Confinados, Seguridad</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v/>
+        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
       </c>
       <c r="B196" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (20 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C196" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Extinción Incendios, Incendios, Seguridad</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v/>
+        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
       </c>
       <c r="B197" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): INSTALACIONES DE TELECOMUNICACIONES</v>
+        <v/>
       </c>
       <c r="C197" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Trabajos en Altura, Seguridad</v>
       </c>
     </row>
     <row r="198">
@@ -2587,367 +2587,191 @@
         <v/>
       </c>
       <c r="B198" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): OPERADORES DE APARATOS ELEVADORES</v>
+        <v>SEGURIDAD Y MANEJO CON PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C198" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>PEMP, Plataformas, Seguridad</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v/>
+        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
       </c>
       <c r="B199" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE ELECTRICIDAD, MONTAJE Y MANTENIMIENTO DE INSTALACIONES DE AT Y BT</v>
+        <v/>
       </c>
       <c r="C199" t="str">
-        <v>Riesgo Eléctrico, Sector Metal, Construcción, Metal, PRL</v>
+        <v>Riesgo Químico, Seguridad</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v/>
+        <v>SEGURIDAD Y SALUD EN TRABAJOS CON RIESGO ELÉCTRICO</v>
       </c>
       <c r="B200" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FERRALLADO</v>
+        <v/>
       </c>
       <c r="C200" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Riesgo Eléctrico, Seguridad</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v/>
+        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
       </c>
       <c r="B201" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE FONTANERÍA E INSTALACIONES DE CLIMATIZACIÓN</v>
+        <v/>
       </c>
       <c r="C201" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>Grúa, Conducción Vehículos</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v/>
+        <v>SOLADOS Y ALICATADOS</v>
       </c>
       <c r="B202" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIÓN DE ASCENSORES</v>
+        <v/>
       </c>
       <c r="C202" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>—</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v/>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
       </c>
       <c r="B203" t="str">
-        <v>SEGUNDO CICLO DE FORMACIÓN EN PRL DEL SECTOR DEL METAL EN OBRAS DE CONSTRUCCIÓN (6 HORAS): TRABAJOS DE INSTALACIONES, REPARACIONES, MONTAJES, ESTRUCTURAS METÁLICAS, CERRAJERÍA Y CARPINTERÍA METÁLICA</v>
+        <v/>
       </c>
       <c r="C203" t="str">
-        <v>Sector Metal, Construcción, Metal, PRL</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>SEGURIDAD EN ANDAMIOS TUBULARES. USO, APLICACIONES Y MONTAJES</v>
+        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
       </c>
       <c r="B204" t="str">
         <v/>
       </c>
       <c r="C204" t="str">
-        <v>Seguridad</v>
+        <v>DEA, Nivel Básico</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS TEORICO - PRACTICO</v>
+        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
       </c>
       <c r="B205" t="str">
         <v/>
       </c>
       <c r="C205" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>SEGURIDAD EN EL USO DE CARRETILLAS ELEVADORAS. RECICLAJE</v>
+        <v/>
       </c>
       <c r="B206" t="str">
-        <v/>
+        <v>TRABAJOS CON RIESGO DE EXPOSICIÓN A FIBRAS DE AMIANTO. TEÓRICO-PRÁCTICO</v>
       </c>
       <c r="C206" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>Amianto</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>SEGURIDAD EN EL USO DE PALA MINICARGADORA</v>
+        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
       </c>
       <c r="B207" t="str">
         <v/>
       </c>
       <c r="C207" t="str">
-        <v>Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>SEGURIDAD EN EL USO DE VEHÍCULOS, TRANSPALETA MANUAL Y APILADOR PARA EL TRANSPORTE Y MANIPULACIÓN DE MERCANCÍAS</v>
+        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
       </c>
       <c r="B208" t="str">
         <v/>
       </c>
       <c r="C208" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>SEGURIDAD EN EN EL USO DE CARRETILLAS ELEVADORAS</v>
+        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
       </c>
       <c r="B209" t="str">
         <v/>
       </c>
       <c r="C209" t="str">
-        <v>Carretillas, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS</v>
+        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
       </c>
       <c r="B210" t="str">
         <v/>
       </c>
       <c r="C210" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL BÁSICO</v>
+        <v>TRABAJOS DE SOLDADURA</v>
       </c>
       <c r="B211" t="str">
         <v/>
       </c>
       <c r="C211" t="str">
-        <v>Espacios Confinados, Nivel Básico, Seguridad</v>
+        <v>Soldadura</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>SEGURIDAD EN ESPACIOS CONFINADOS: NIVEL INICIACIÓN</v>
+        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
       </c>
       <c r="B212" t="str">
         <v/>
       </c>
       <c r="C212" t="str">
-        <v>Espacios Confinados, Seguridad</v>
+        <v>Trabajos en Altura</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>SEGURIDAD EN LA EXTINCIÓN DE INCENDIOS</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
       </c>
       <c r="B213" t="str">
         <v/>
       </c>
       <c r="C213" t="str">
-        <v>Extinción Incendios, Incendios, Seguridad</v>
+        <v>—</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ALTURA: NIVEL INICIACIÓN</v>
+        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
       </c>
       <c r="B214" t="str">
         <v/>
       </c>
       <c r="C214" t="str">
-        <v>Trabajos en Altura, Seguridad</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="str">
-        <v/>
-      </c>
-      <c r="B215" t="str">
-        <v>SEGURIDAD EN TRABAJOS EN ESAPCIOS CONFINADOS. NIVEL 1. TEÓRICO-PRÁCTICO</v>
-      </c>
-      <c r="C215" t="str">
-        <v>Seguridad</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="str">
-        <v/>
-      </c>
-      <c r="B216" t="str">
-        <v>SEGURIDAD Y MANEJO CON PLATAFORMAS ELEVADORAS. TEÓRICO-PRÁCTICO</v>
-      </c>
-      <c r="C216" t="str">
-        <v>PEMP, Plataformas, Seguridad</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="str">
-        <v>SEGURIDAD Y SALUD EN EL MANEJO DE PRODUCTOS QUÍMICOS</v>
-      </c>
-      <c r="B217" t="str">
-        <v/>
-      </c>
-      <c r="C217" t="str">
-        <v>Riesgo Químico, Seguridad</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="str">
-        <v>SEÑALISTA-ESLINGADOR PARA MANIOBRAS DE GRÚAS AUTOPROPULSADAS Y CAMIONES GRÚAS</v>
-      </c>
-      <c r="B218" t="str">
-        <v/>
-      </c>
-      <c r="C218" t="str">
-        <v>Grúa, Conducción Vehículos</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="str">
-        <v>SOLADOS Y ALICATADOS</v>
-      </c>
-      <c r="B219" t="str">
-        <v/>
-      </c>
-      <c r="C219" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR</v>
-      </c>
-      <c r="B220" t="str">
-        <v/>
-      </c>
-      <c r="C220" t="str">
-        <v>DEA, Nivel Básico</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="str">
-        <v>SOPORTE VITAL BÁSICO Y USO DE DESFIBRILADOR SEGÚN ACREDITACIÓN CCR</v>
-      </c>
-      <c r="B221" t="str">
-        <v/>
-      </c>
-      <c r="C221" t="str">
-        <v>DEA, Nivel Básico</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="str">
-        <v>TALLERES DE REPARACIÓN DE VEHÍCULOS</v>
-      </c>
-      <c r="B222" t="str">
-        <v/>
-      </c>
-      <c r="C222" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="str">
-        <v>TRABAJOS DE AISLAMIENTO E IMPERMEABILIZACIÓN</v>
-      </c>
-      <c r="B223" t="str">
-        <v/>
-      </c>
-      <c r="C223" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="str">
-        <v>TRABAJOS DE MONTAJE DE ESTRUCTURAS TUBULARES</v>
-      </c>
-      <c r="B224" t="str">
-        <v/>
-      </c>
-      <c r="C224" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="str">
-        <v>TRABAJOS DE MONTAJE DE PREFABRICADOS DE HORMIGÓN EN OBRA</v>
-      </c>
-      <c r="B225" t="str">
-        <v/>
-      </c>
-      <c r="C225" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="str">
-        <v>TRABAJOS DE REDES DE ABASTECIMIENTO Y SANEAMIENTO Y POCERÍA</v>
-      </c>
-      <c r="B226" t="str">
-        <v/>
-      </c>
-      <c r="C226" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="str">
-        <v>TRABAJOS DE SOLDADURA</v>
-      </c>
-      <c r="B227" t="str">
-        <v/>
-      </c>
-      <c r="C227" t="str">
-        <v>Soldadura</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="str">
-        <v>TRABAJOS EN ALTURA CON PROTECCIÓN INDIVIDUAL</v>
-      </c>
-      <c r="B228" t="str">
-        <v/>
-      </c>
-      <c r="C228" t="str">
-        <v>Trabajos en Altura</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE RÓTULOS</v>
-      </c>
-      <c r="B229" t="str">
-        <v/>
-      </c>
-      <c r="C229" t="str">
-        <v>—</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="str">
-        <v>VIDRIO Y ROTULACIÓN: INSTALADOR DE VENTANAS Y ACRISTALAMIENTOS</v>
-      </c>
-      <c r="B230" t="str">
-        <v/>
-      </c>
-      <c r="C230" t="str">
         <v>—</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C214"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>